<commit_message>
Refactor avatar components and styles across multiple pages
- Replaced q-avatar components with custom portrait badges in CompaniesPage, NotesPage, OpportunitiesPage, ProjectsPage, TasksPage, and UsersPage.
- Updated avatar color and initial generation logic for better consistency.
- Enhanced toolbar styles for better alignment and appearance.
- Removed unused avatar building functions and optimized CSS for card components.
- Introduced new environment configuration for Electron development.
</commit_message>
<xml_diff>
--- a/docs/B10_DOS v260400 vrev.xlsx
+++ b/docs/B10_DOS v260400 vrev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erikc\Coding_Repository\ec-vc\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B705EE4-DC10-452F-8F60-401889F147CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C6F546D-CD95-498D-AA7B-6E620C399E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{0110398B-6F4E-42D1-8445-B061DE6C3E3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0110398B-6F4E-42D1-8445-B061DE6C3E3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokens" sheetId="1" r:id="rId1"/>
@@ -2231,7 +2231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:O1097"/>
@@ -2239,10 +2239,10 @@
   <cols>
     <col min="1" max="1" width="2.85546875" customWidth="1"/>
     <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="7.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="7.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="11.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="7" max="7" width="14.28515625" customWidth="1" outlineLevel="1"/>
     <col min="8" max="8" width="20.28515625" customWidth="1" outlineLevel="1"/>
     <col min="9" max="9" width="29.42578125" style="18" bestFit="1" customWidth="1"/>
@@ -2349,7 +2349,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="31">
         <v>1</v>
@@ -2394,7 +2394,7 @@
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
     </row>
-    <row r="7" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="31">
         <f>+B6+1</f>
@@ -2440,7 +2440,7 @@
       <c r="N7" s="9"/>
       <c r="O7" s="9"/>
     </row>
-    <row r="8" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="31">
         <f t="shared" ref="B8:B71" si="3">+B7+1</f>
@@ -2486,7 +2486,7 @@
       <c r="N8" s="9"/>
       <c r="O8" s="9"/>
     </row>
-    <row r="9" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="31">
         <f t="shared" si="3"/>
@@ -2532,7 +2532,7 @@
       <c r="N9" s="9"/>
       <c r="O9" s="9"/>
     </row>
-    <row r="10" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="31">
         <f t="shared" si="3"/>
@@ -2578,7 +2578,7 @@
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
     </row>
-    <row r="11" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="31">
         <f t="shared" si="3"/>
@@ -2624,7 +2624,7 @@
       <c r="N11" s="9"/>
       <c r="O11" s="9"/>
     </row>
-    <row r="12" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="31">
         <f t="shared" si="3"/>
@@ -2670,7 +2670,7 @@
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
     </row>
-    <row r="13" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="31">
         <f t="shared" si="3"/>
@@ -2716,7 +2716,7 @@
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
     </row>
-    <row r="14" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="31">
         <f t="shared" si="3"/>
@@ -2762,7 +2762,7 @@
       <c r="N14" s="9"/>
       <c r="O14" s="9"/>
     </row>
-    <row r="15" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="31">
         <f t="shared" si="3"/>
@@ -2808,7 +2808,7 @@
       <c r="N15" s="9"/>
       <c r="O15" s="9"/>
     </row>
-    <row r="16" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="31">
         <f t="shared" si="3"/>
@@ -2854,7 +2854,7 @@
       <c r="N16" s="9"/>
       <c r="O16" s="9"/>
     </row>
-    <row r="17" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="31">
         <f t="shared" si="3"/>
@@ -2900,7 +2900,7 @@
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
     </row>
-    <row r="18" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="31">
         <f t="shared" si="3"/>
@@ -2946,7 +2946,7 @@
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
     </row>
-    <row r="19" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
       <c r="B19" s="31">
         <f t="shared" si="3"/>
@@ -2992,7 +2992,7 @@
       <c r="N19" s="9"/>
       <c r="O19" s="9"/>
     </row>
-    <row r="20" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="31">
         <f t="shared" si="3"/>
@@ -3038,7 +3038,7 @@
       <c r="N20" s="9"/>
       <c r="O20" s="9"/>
     </row>
-    <row r="21" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="31">
         <f t="shared" si="3"/>
@@ -3084,7 +3084,7 @@
       <c r="N21" s="9"/>
       <c r="O21" s="9"/>
     </row>
-    <row r="22" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="31">
         <f t="shared" si="3"/>
@@ -3130,7 +3130,7 @@
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
     </row>
-    <row r="23" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="31">
         <f t="shared" si="3"/>
@@ -3176,7 +3176,7 @@
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
     </row>
-    <row r="24" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="31">
         <f t="shared" si="3"/>
@@ -3222,7 +3222,7 @@
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
     </row>
-    <row r="25" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="31">
         <f t="shared" si="3"/>
@@ -3268,7 +3268,7 @@
       <c r="N25" s="9"/>
       <c r="O25" s="9"/>
     </row>
-    <row r="26" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
       <c r="B26" s="31">
         <f t="shared" si="3"/>
@@ -3314,7 +3314,7 @@
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
     </row>
-    <row r="27" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8"/>
       <c r="B27" s="31">
         <f t="shared" si="3"/>
@@ -3360,7 +3360,7 @@
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
     </row>
-    <row r="28" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8"/>
       <c r="B28" s="31">
         <f t="shared" si="3"/>
@@ -3406,7 +3406,7 @@
       <c r="N28" s="9"/>
       <c r="O28" s="9"/>
     </row>
-    <row r="29" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" s="31">
         <f t="shared" si="3"/>
@@ -3452,7 +3452,7 @@
       <c r="N29" s="9"/>
       <c r="O29" s="9"/>
     </row>
-    <row r="30" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
       <c r="B30" s="31">
         <f t="shared" si="3"/>
@@ -3498,7 +3498,7 @@
       <c r="N30" s="9"/>
       <c r="O30" s="9"/>
     </row>
-    <row r="31" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
       <c r="B31" s="31">
         <f t="shared" si="3"/>
@@ -3544,7 +3544,7 @@
       <c r="N31" s="9"/>
       <c r="O31" s="9"/>
     </row>
-    <row r="32" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8"/>
       <c r="B32" s="31">
         <f t="shared" si="3"/>
@@ -3590,7 +3590,7 @@
       <c r="N32" s="9"/>
       <c r="O32" s="9"/>
     </row>
-    <row r="33" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
       <c r="B33" s="31">
         <f t="shared" si="3"/>
@@ -3636,7 +3636,7 @@
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
     </row>
-    <row r="34" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
       <c r="B34" s="31">
         <f t="shared" si="3"/>
@@ -3682,7 +3682,7 @@
       <c r="N34" s="9"/>
       <c r="O34" s="9"/>
     </row>
-    <row r="35" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="31">
         <f t="shared" si="3"/>
@@ -3728,7 +3728,7 @@
       <c r="N35" s="9"/>
       <c r="O35" s="9"/>
     </row>
-    <row r="36" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8"/>
       <c r="B36" s="31">
         <f t="shared" si="3"/>
@@ -3774,7 +3774,7 @@
       <c r="N36" s="9"/>
       <c r="O36" s="9"/>
     </row>
-    <row r="37" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8"/>
       <c r="B37" s="31">
         <f t="shared" si="3"/>
@@ -3820,7 +3820,7 @@
       <c r="N37" s="9"/>
       <c r="O37" s="9"/>
     </row>
-    <row r="38" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8"/>
       <c r="B38" s="31">
         <f t="shared" si="3"/>
@@ -3866,7 +3866,7 @@
       <c r="N38" s="9"/>
       <c r="O38" s="9"/>
     </row>
-    <row r="39" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="31">
         <f t="shared" si="3"/>
@@ -3912,7 +3912,7 @@
       <c r="N39" s="9"/>
       <c r="O39" s="9"/>
     </row>
-    <row r="40" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8"/>
       <c r="B40" s="31">
         <f t="shared" si="3"/>
@@ -3958,7 +3958,7 @@
       <c r="N40" s="9"/>
       <c r="O40" s="9"/>
     </row>
-    <row r="41" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
       <c r="B41" s="31">
         <f t="shared" si="3"/>
@@ -4004,7 +4004,7 @@
       <c r="N41" s="9"/>
       <c r="O41" s="9"/>
     </row>
-    <row r="42" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
       <c r="B42" s="31">
         <f t="shared" si="3"/>
@@ -4050,7 +4050,7 @@
       <c r="N42" s="9"/>
       <c r="O42" s="9"/>
     </row>
-    <row r="43" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="31">
         <f t="shared" si="3"/>
@@ -4096,7 +4096,7 @@
       <c r="N43" s="9"/>
       <c r="O43" s="9"/>
     </row>
-    <row r="44" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
       <c r="B44" s="31">
         <f t="shared" si="3"/>
@@ -4142,7 +4142,7 @@
       <c r="N44" s="9"/>
       <c r="O44" s="9"/>
     </row>
-    <row r="45" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
       <c r="B45" s="31">
         <f t="shared" si="3"/>
@@ -4188,7 +4188,7 @@
       <c r="N45" s="9"/>
       <c r="O45" s="9"/>
     </row>
-    <row r="46" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>
       <c r="B46" s="31">
         <f t="shared" si="3"/>
@@ -4234,7 +4234,7 @@
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
     </row>
-    <row r="47" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
       <c r="B47" s="31">
         <f t="shared" si="3"/>
@@ -4280,7 +4280,7 @@
       <c r="N47" s="9"/>
       <c r="O47" s="1"/>
     </row>
-    <row r="48" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="31">
         <f t="shared" si="3"/>
@@ -4326,7 +4326,7 @@
       <c r="N48" s="9"/>
       <c r="O48" s="1"/>
     </row>
-    <row r="49" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="31">
         <f t="shared" si="3"/>
@@ -4372,7 +4372,7 @@
       <c r="N49" s="9"/>
       <c r="O49" s="1"/>
     </row>
-    <row r="50" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="31">
         <f t="shared" si="3"/>
@@ -4418,7 +4418,7 @@
       <c r="N50" s="9"/>
       <c r="O50" s="1"/>
     </row>
-    <row r="51" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A51" s="8"/>
       <c r="B51" s="31">
         <f t="shared" si="3"/>
@@ -4464,7 +4464,7 @@
       <c r="N51" s="9"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A52" s="8"/>
       <c r="B52" s="31">
         <f t="shared" si="3"/>
@@ -4510,7 +4510,7 @@
       <c r="N52" s="9"/>
       <c r="O52" s="1"/>
     </row>
-    <row r="53" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
       <c r="B53" s="31">
         <f t="shared" si="3"/>
@@ -4556,7 +4556,7 @@
       <c r="N53" s="9"/>
       <c r="O53" s="1"/>
     </row>
-    <row r="54" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
       <c r="B54" s="31">
         <f t="shared" si="3"/>
@@ -4602,7 +4602,7 @@
       <c r="N54" s="9"/>
       <c r="O54" s="1"/>
     </row>
-    <row r="55" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8"/>
       <c r="B55" s="31">
         <f t="shared" si="3"/>
@@ -4648,7 +4648,7 @@
       <c r="N55" s="9"/>
       <c r="O55" s="9"/>
     </row>
-    <row r="56" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8"/>
       <c r="B56" s="31">
         <f t="shared" si="3"/>
@@ -4694,7 +4694,7 @@
       <c r="N56" s="9"/>
       <c r="O56" s="9"/>
     </row>
-    <row r="57" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8"/>
       <c r="B57" s="31">
         <f t="shared" si="3"/>
@@ -4740,7 +4740,7 @@
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
     </row>
-    <row r="58" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8"/>
       <c r="B58" s="31">
         <f t="shared" si="3"/>
@@ -4786,7 +4786,7 @@
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
     </row>
-    <row r="59" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8"/>
       <c r="B59" s="31">
         <f t="shared" si="3"/>
@@ -4832,7 +4832,7 @@
       <c r="N59" s="9"/>
       <c r="O59" s="9"/>
     </row>
-    <row r="60" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8"/>
       <c r="B60" s="31">
         <f t="shared" si="3"/>
@@ -4878,7 +4878,7 @@
       <c r="N60" s="9"/>
       <c r="O60" s="9"/>
     </row>
-    <row r="61" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8"/>
       <c r="B61" s="31">
         <f t="shared" si="3"/>
@@ -4924,7 +4924,7 @@
       <c r="N61" s="9"/>
       <c r="O61" s="9"/>
     </row>
-    <row r="62" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8"/>
       <c r="B62" s="31">
         <f t="shared" si="3"/>
@@ -4970,7 +4970,7 @@
       <c r="N62" s="9"/>
       <c r="O62" s="9"/>
     </row>
-    <row r="63" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8"/>
       <c r="B63" s="31">
         <f t="shared" si="3"/>
@@ -5016,7 +5016,7 @@
       <c r="N63" s="9"/>
       <c r="O63" s="9"/>
     </row>
-    <row r="64" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A64" s="8"/>
       <c r="B64" s="31">
         <f t="shared" si="3"/>
@@ -5062,7 +5062,7 @@
       <c r="N64" s="9"/>
       <c r="O64" s="1"/>
     </row>
-    <row r="65" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
       <c r="B65" s="31">
         <f t="shared" si="3"/>
@@ -5108,7 +5108,7 @@
       <c r="N65" s="9"/>
       <c r="O65" s="1"/>
     </row>
-    <row r="66" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A66" s="8"/>
       <c r="B66" s="31">
         <f t="shared" si="3"/>
@@ -5154,7 +5154,7 @@
       <c r="N66" s="9"/>
       <c r="O66" s="1"/>
     </row>
-    <row r="67" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A67" s="8"/>
       <c r="B67" s="31">
         <f t="shared" si="3"/>
@@ -5200,7 +5200,7 @@
       <c r="N67" s="9"/>
       <c r="O67" s="1"/>
     </row>
-    <row r="68" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A68" s="8"/>
       <c r="B68" s="31">
         <f t="shared" si="3"/>
@@ -5246,7 +5246,7 @@
       <c r="N68" s="9"/>
       <c r="O68" s="1"/>
     </row>
-    <row r="69" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A69" s="8"/>
       <c r="B69" s="31">
         <f t="shared" si="3"/>
@@ -5292,7 +5292,7 @@
       <c r="N69" s="9"/>
       <c r="O69" s="1"/>
     </row>
-    <row r="70" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A70" s="8"/>
       <c r="B70" s="31">
         <f t="shared" si="3"/>
@@ -5338,7 +5338,7 @@
       <c r="N70" s="9"/>
       <c r="O70" s="1"/>
     </row>
-    <row r="71" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A71" s="8"/>
       <c r="B71" s="31">
         <f t="shared" si="3"/>
@@ -5384,7 +5384,7 @@
       <c r="N71" s="9"/>
       <c r="O71" s="1"/>
     </row>
-    <row r="72" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A72" s="8"/>
       <c r="B72" s="31">
         <f t="shared" ref="B72:B136" si="35">+B71+1</f>
@@ -5430,7 +5430,7 @@
       <c r="N72" s="9"/>
       <c r="O72" s="1"/>
     </row>
-    <row r="73" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A73" s="8"/>
       <c r="B73" s="31">
         <f t="shared" si="35"/>
@@ -5476,7 +5476,7 @@
       <c r="N73" s="9"/>
       <c r="O73" s="1"/>
     </row>
-    <row r="74" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A74" s="8"/>
       <c r="B74" s="31">
         <f t="shared" si="35"/>
@@ -5522,7 +5522,7 @@
       <c r="N74" s="9"/>
       <c r="O74" s="1"/>
     </row>
-    <row r="75" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
       <c r="B75" s="31">
         <f t="shared" si="35"/>
@@ -5568,7 +5568,7 @@
       <c r="N75" s="9"/>
       <c r="O75" s="1"/>
     </row>
-    <row r="76" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A76" s="8"/>
       <c r="B76" s="31">
         <f t="shared" si="35"/>
@@ -5614,7 +5614,7 @@
       <c r="N76" s="9"/>
       <c r="O76" s="1"/>
     </row>
-    <row r="77" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A77" s="8"/>
       <c r="B77" s="31">
         <f t="shared" si="35"/>
@@ -5660,7 +5660,7 @@
       <c r="N77" s="9"/>
       <c r="O77" s="1"/>
     </row>
-    <row r="78" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A78" s="8"/>
       <c r="B78" s="31">
         <f t="shared" si="35"/>
@@ -5706,7 +5706,7 @@
       <c r="N78" s="9"/>
       <c r="O78" s="1"/>
     </row>
-    <row r="79" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A79" s="8"/>
       <c r="B79" s="31">
         <f t="shared" si="35"/>
@@ -5752,7 +5752,7 @@
       <c r="N79" s="9"/>
       <c r="O79" s="1"/>
     </row>
-    <row r="80" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A80" s="8"/>
       <c r="B80" s="31">
         <f t="shared" si="35"/>
@@ -5798,7 +5798,7 @@
       <c r="N80" s="9"/>
       <c r="O80" s="1"/>
     </row>
-    <row r="81" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A81" s="8"/>
       <c r="B81" s="31">
         <f t="shared" si="35"/>
@@ -5844,7 +5844,7 @@
       <c r="N81" s="9"/>
       <c r="O81" s="1"/>
     </row>
-    <row r="82" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A82" s="8"/>
       <c r="B82" s="31">
         <f t="shared" si="35"/>
@@ -5890,7 +5890,7 @@
       <c r="N82" s="9"/>
       <c r="O82" s="1"/>
     </row>
-    <row r="83" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A83" s="8"/>
       <c r="B83" s="31">
         <f t="shared" si="35"/>
@@ -5936,7 +5936,7 @@
       <c r="N83" s="9"/>
       <c r="O83" s="1"/>
     </row>
-    <row r="84" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A84" s="8"/>
       <c r="B84" s="31">
         <f t="shared" si="35"/>
@@ -5982,7 +5982,7 @@
       <c r="N84" s="9"/>
       <c r="O84" s="1"/>
     </row>
-    <row r="85" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A85" s="8"/>
       <c r="B85" s="31">
         <f t="shared" si="35"/>
@@ -6028,7 +6028,7 @@
       <c r="N85" s="9"/>
       <c r="O85" s="1"/>
     </row>
-    <row r="86" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A86" s="8"/>
       <c r="B86" s="31">
         <f t="shared" si="35"/>
@@ -6074,7 +6074,7 @@
       <c r="N86" s="9"/>
       <c r="O86" s="1"/>
     </row>
-    <row r="87" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A87" s="8"/>
       <c r="B87" s="31">
         <f t="shared" si="35"/>
@@ -6120,7 +6120,7 @@
       <c r="N87" s="9"/>
       <c r="O87" s="1"/>
     </row>
-    <row r="88" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A88" s="8"/>
       <c r="B88" s="31">
         <f t="shared" si="35"/>
@@ -6166,7 +6166,7 @@
       <c r="N88" s="9"/>
       <c r="O88" s="1"/>
     </row>
-    <row r="89" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A89" s="8"/>
       <c r="B89" s="31">
         <f t="shared" si="35"/>
@@ -6212,7 +6212,7 @@
       <c r="N89" s="9"/>
       <c r="O89" s="1"/>
     </row>
-    <row r="90" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A90" s="8"/>
       <c r="B90" s="31">
         <f t="shared" si="35"/>
@@ -6258,7 +6258,7 @@
       <c r="N90" s="9"/>
       <c r="O90" s="1"/>
     </row>
-    <row r="91" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A91" s="8"/>
       <c r="B91" s="31">
         <f t="shared" si="35"/>
@@ -6304,7 +6304,7 @@
       <c r="N91" s="9"/>
       <c r="O91" s="1"/>
     </row>
-    <row r="92" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A92" s="8"/>
       <c r="B92" s="31">
         <f t="shared" si="35"/>
@@ -6350,7 +6350,7 @@
       <c r="N92" s="9"/>
       <c r="O92" s="1"/>
     </row>
-    <row r="93" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A93" s="8"/>
       <c r="B93" s="31">
         <f t="shared" si="35"/>
@@ -6396,7 +6396,7 @@
       <c r="N93" s="9"/>
       <c r="O93" s="1"/>
     </row>
-    <row r="94" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A94" s="8"/>
       <c r="B94" s="31">
         <f t="shared" si="35"/>
@@ -6442,7 +6442,7 @@
       <c r="N94" s="9"/>
       <c r="O94" s="1"/>
     </row>
-    <row r="95" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A95" s="8"/>
       <c r="B95" s="31">
         <f t="shared" si="35"/>
@@ -6488,7 +6488,7 @@
       <c r="N95" s="9"/>
       <c r="O95" s="1"/>
     </row>
-    <row r="96" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A96" s="8"/>
       <c r="B96" s="31">
         <f t="shared" si="35"/>
@@ -6534,7 +6534,7 @@
       <c r="N96" s="9"/>
       <c r="O96" s="1"/>
     </row>
-    <row r="97" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A97" s="8"/>
       <c r="B97" s="31">
         <f t="shared" si="35"/>
@@ -6580,7 +6580,7 @@
       <c r="N97" s="9"/>
       <c r="O97" s="1"/>
     </row>
-    <row r="98" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A98" s="8"/>
       <c r="B98" s="31">
         <f t="shared" si="35"/>
@@ -6626,7 +6626,7 @@
       <c r="N98" s="9"/>
       <c r="O98" s="1"/>
     </row>
-    <row r="99" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A99" s="8"/>
       <c r="B99" s="31">
         <f t="shared" si="35"/>
@@ -6672,7 +6672,7 @@
       <c r="N99" s="9"/>
       <c r="O99" s="1"/>
     </row>
-    <row r="100" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A100" s="8"/>
       <c r="B100" s="31">
         <f t="shared" si="35"/>
@@ -6718,7 +6718,7 @@
       <c r="N100" s="9"/>
       <c r="O100" s="1"/>
     </row>
-    <row r="101" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A101" s="8"/>
       <c r="B101" s="31">
         <f t="shared" ref="B101:B102" si="41">+B100+1</f>
@@ -6764,7 +6764,7 @@
       <c r="N101" s="9"/>
       <c r="O101" s="1"/>
     </row>
-    <row r="102" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A102" s="8"/>
       <c r="B102" s="31">
         <f t="shared" si="41"/>
@@ -6810,7 +6810,7 @@
       <c r="N102" s="9"/>
       <c r="O102" s="1"/>
     </row>
-    <row r="103" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A103" s="8"/>
       <c r="B103" s="31">
         <f t="shared" si="35"/>
@@ -6856,7 +6856,7 @@
       <c r="N103" s="9"/>
       <c r="O103" s="1"/>
     </row>
-    <row r="104" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A104" s="8"/>
       <c r="B104" s="31">
         <f t="shared" si="35"/>
@@ -6902,7 +6902,7 @@
       <c r="N104" s="9"/>
       <c r="O104" s="1"/>
     </row>
-    <row r="105" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A105" s="8"/>
       <c r="B105" s="31">
         <f t="shared" si="35"/>
@@ -6948,7 +6948,7 @@
       <c r="N105" s="9"/>
       <c r="O105" s="1"/>
     </row>
-    <row r="106" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A106" s="8"/>
       <c r="B106" s="31">
         <f t="shared" si="35"/>
@@ -6994,7 +6994,7 @@
       <c r="N106" s="9"/>
       <c r="O106" s="1"/>
     </row>
-    <row r="107" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A107" s="8"/>
       <c r="B107" s="31">
         <f t="shared" si="35"/>
@@ -7040,7 +7040,7 @@
       <c r="N107" s="9"/>
       <c r="O107" s="1"/>
     </row>
-    <row r="108" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A108" s="8"/>
       <c r="B108" s="31">
         <f t="shared" si="35"/>
@@ -7086,7 +7086,7 @@
       <c r="N108" s="9"/>
       <c r="O108" s="1"/>
     </row>
-    <row r="109" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A109" s="8"/>
       <c r="B109" s="31">
         <f t="shared" si="35"/>
@@ -7132,7 +7132,7 @@
       <c r="N109" s="9"/>
       <c r="O109" s="1"/>
     </row>
-    <row r="110" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A110" s="8"/>
       <c r="B110" s="31">
         <f t="shared" si="35"/>
@@ -7178,7 +7178,7 @@
       <c r="N110" s="9"/>
       <c r="O110" s="1"/>
     </row>
-    <row r="111" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A111" s="8"/>
       <c r="B111" s="31">
         <f t="shared" si="35"/>
@@ -7224,7 +7224,7 @@
       <c r="N111" s="9"/>
       <c r="O111" s="1"/>
     </row>
-    <row r="112" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A112" s="8"/>
       <c r="B112" s="31">
         <f t="shared" si="35"/>
@@ -7270,7 +7270,7 @@
       <c r="N112" s="9"/>
       <c r="O112" s="1"/>
     </row>
-    <row r="113" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A113" s="8"/>
       <c r="B113" s="31">
         <f t="shared" si="35"/>
@@ -7316,7 +7316,7 @@
       <c r="N113" s="9"/>
       <c r="O113" s="1"/>
     </row>
-    <row r="114" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A114" s="8"/>
       <c r="B114" s="31">
         <f t="shared" si="35"/>
@@ -7362,7 +7362,7 @@
       <c r="N114" s="9"/>
       <c r="O114" s="1"/>
     </row>
-    <row r="115" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A115" s="8"/>
       <c r="B115" s="31">
         <f t="shared" si="35"/>
@@ -7408,7 +7408,7 @@
       <c r="N115" s="9"/>
       <c r="O115" s="1"/>
     </row>
-    <row r="116" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A116" s="8"/>
       <c r="B116" s="31">
         <f t="shared" si="35"/>
@@ -7454,7 +7454,7 @@
       <c r="N116" s="9"/>
       <c r="O116" s="1"/>
     </row>
-    <row r="117" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A117" s="8"/>
       <c r="B117" s="31">
         <f t="shared" si="35"/>
@@ -7500,7 +7500,7 @@
       <c r="N117" s="9"/>
       <c r="O117" s="1"/>
     </row>
-    <row r="118" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A118" s="8"/>
       <c r="B118" s="31">
         <f t="shared" si="35"/>
@@ -7546,7 +7546,7 @@
       <c r="N118" s="9"/>
       <c r="O118" s="1"/>
     </row>
-    <row r="119" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A119" s="8"/>
       <c r="B119" s="31">
         <f t="shared" si="35"/>
@@ -7592,7 +7592,7 @@
       <c r="N119" s="9"/>
       <c r="O119" s="1"/>
     </row>
-    <row r="120" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A120" s="8"/>
       <c r="B120" s="31">
         <f t="shared" si="35"/>
@@ -7638,7 +7638,7 @@
       <c r="N120" s="9"/>
       <c r="O120" s="1"/>
     </row>
-    <row r="121" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A121" s="8"/>
       <c r="B121" s="31">
         <f t="shared" si="35"/>
@@ -7684,7 +7684,7 @@
       <c r="N121" s="9"/>
       <c r="O121" s="1"/>
     </row>
-    <row r="122" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8"/>
       <c r="B122" s="31">
         <f t="shared" si="35"/>
@@ -7730,7 +7730,7 @@
       <c r="N122" s="9"/>
       <c r="O122" s="1"/>
     </row>
-    <row r="123" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A123" s="8"/>
       <c r="B123" s="31">
         <f t="shared" si="35"/>
@@ -7776,7 +7776,7 @@
       <c r="N123" s="9"/>
       <c r="O123" s="1"/>
     </row>
-    <row r="124" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A124" s="8"/>
       <c r="B124" s="31">
         <f t="shared" si="35"/>
@@ -7822,7 +7822,7 @@
       <c r="N124" s="9"/>
       <c r="O124" s="1"/>
     </row>
-    <row r="125" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A125" s="8"/>
       <c r="B125" s="31">
         <f t="shared" si="35"/>
@@ -7868,7 +7868,7 @@
       <c r="N125" s="9"/>
       <c r="O125" s="1"/>
     </row>
-    <row r="126" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A126" s="8"/>
       <c r="B126" s="31">
         <f t="shared" si="35"/>
@@ -7914,7 +7914,7 @@
       <c r="N126" s="9"/>
       <c r="O126" s="1"/>
     </row>
-    <row r="127" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A127" s="8"/>
       <c r="B127" s="31">
         <f t="shared" si="35"/>
@@ -7960,7 +7960,7 @@
       <c r="N127" s="9"/>
       <c r="O127" s="1"/>
     </row>
-    <row r="128" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A128" s="8"/>
       <c r="B128" s="31">
         <f t="shared" si="35"/>
@@ -8006,7 +8006,7 @@
       <c r="N128" s="9"/>
       <c r="O128" s="1"/>
     </row>
-    <row r="129" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A129" s="8"/>
       <c r="B129" s="31">
         <f t="shared" si="35"/>
@@ -8052,7 +8052,7 @@
       <c r="N129" s="9"/>
       <c r="O129" s="1"/>
     </row>
-    <row r="130" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A130" s="8"/>
       <c r="B130" s="31">
         <f t="shared" si="35"/>
@@ -8098,7 +8098,7 @@
       <c r="N130" s="9"/>
       <c r="O130" s="1"/>
     </row>
-    <row r="131" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A131" s="8"/>
       <c r="B131" s="31">
         <f t="shared" si="35"/>
@@ -8144,7 +8144,7 @@
       <c r="N131" s="9"/>
       <c r="O131" s="1"/>
     </row>
-    <row r="132" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A132" s="8"/>
       <c r="B132" s="31">
         <f t="shared" si="35"/>
@@ -8190,7 +8190,7 @@
       <c r="N132" s="9"/>
       <c r="O132" s="1"/>
     </row>
-    <row r="133" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A133" s="8"/>
       <c r="B133" s="31">
         <f t="shared" si="35"/>
@@ -8236,7 +8236,7 @@
       <c r="N133" s="9"/>
       <c r="O133" s="1"/>
     </row>
-    <row r="134" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
       <c r="B134" s="31">
         <f t="shared" si="35"/>
@@ -9306,21 +9306,21 @@
       </c>
       <c r="D157" s="24">
         <f t="shared" ref="D157" si="64">((C157&lt;&gt;C156)*1)+((C157=C156)*(H157=H156)*(D156))+((C157=C156)*(H157&lt;&gt;H156)*(D156+1))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E157" s="24">
         <f t="shared" ref="E157" si="65">((H157&lt;&gt;H156)*1)+((H157=H156)*(E156+1))</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F157" s="32" t="str">
         <f>_xlfn.CONCAT(C157,".",D157,".",E157)</f>
-        <v>5.4.1</v>
+        <v>5.3.9</v>
       </c>
       <c r="G157" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H157" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I157" s="19" t="s">
         <v>304</v>
@@ -9352,21 +9352,21 @@
       </c>
       <c r="D158" s="24">
         <f t="shared" ref="D158:D161" si="66">((C158&lt;&gt;C157)*1)+((C158=C157)*(H158=H157)*(D157))+((C158=C157)*(H158&lt;&gt;H157)*(D157+1))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E158" s="24">
         <f t="shared" ref="E158:E161" si="67">((H158&lt;&gt;H157)*1)+((H158=H157)*(E157+1))</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F158" s="32" t="str">
         <f t="shared" ref="F158:F161" si="68">_xlfn.CONCAT(C158,".",D158,".",E158)</f>
-        <v>5.4.2</v>
+        <v>5.3.10</v>
       </c>
       <c r="G158" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H158" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I158" s="19" t="s">
         <v>79</v>
@@ -9398,21 +9398,21 @@
       </c>
       <c r="D159" s="24">
         <f t="shared" si="66"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E159" s="24">
         <f t="shared" si="67"/>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F159" s="32" t="str">
         <f t="shared" si="68"/>
-        <v>5.4.3</v>
+        <v>5.3.11</v>
       </c>
       <c r="G159" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H159" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I159" s="19" t="s">
         <v>80</v>
@@ -9444,21 +9444,21 @@
       </c>
       <c r="D160" s="24">
         <f t="shared" si="66"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E160" s="24">
         <f t="shared" si="67"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F160" s="32" t="str">
         <f t="shared" si="68"/>
-        <v>5.4.4</v>
+        <v>5.3.12</v>
       </c>
       <c r="G160" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H160" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I160" s="19" t="s">
         <v>161</v>
@@ -9490,21 +9490,21 @@
       </c>
       <c r="D161" s="24">
         <f t="shared" si="66"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E161" s="24">
         <f t="shared" si="67"/>
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F161" s="32" t="str">
         <f t="shared" si="68"/>
-        <v>5.4.5</v>
+        <v>5.3.13</v>
       </c>
       <c r="G161" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H161" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I161" s="19" t="s">
         <v>162</v>
@@ -9536,21 +9536,21 @@
       </c>
       <c r="D162" s="24">
         <f t="shared" ref="D162:D164" si="69">((C162&lt;&gt;C161)*1)+((C162=C161)*(H162=H161)*(D161))+((C162=C161)*(H162&lt;&gt;H161)*(D161+1))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E162" s="24">
         <f t="shared" ref="E162:E164" si="70">((H162&lt;&gt;H161)*1)+((H162=H161)*(E161+1))</f>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F162" s="32" t="str">
         <f>_xlfn.CONCAT(C162,".",D162,".",E162)</f>
-        <v>5.4.6</v>
+        <v>5.3.14</v>
       </c>
       <c r="G162" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H162" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I162" s="19" t="s">
         <v>164</v>
@@ -9582,21 +9582,21 @@
       </c>
       <c r="D163" s="24">
         <f t="shared" si="69"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E163" s="24">
         <f t="shared" si="70"/>
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F163" s="32" t="str">
         <f>_xlfn.CONCAT(C163,".",D163,".",E163)</f>
-        <v>5.4.7</v>
+        <v>5.3.15</v>
       </c>
       <c r="G163" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H163" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I163" s="19" t="s">
         <v>165</v>
@@ -9628,21 +9628,21 @@
       </c>
       <c r="D164" s="24">
         <f t="shared" si="69"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E164" s="24">
         <f t="shared" si="70"/>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F164" s="32" t="str">
         <f>_xlfn.CONCAT(C164,".",D164,".",E164)</f>
-        <v>5.4.8</v>
+        <v>5.3.16</v>
       </c>
       <c r="G164" s="19" t="s">
         <v>573</v>
       </c>
       <c r="H164" s="19" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="I164" s="19" t="s">
         <v>305</v>
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D165" s="24">
         <f t="shared" ref="D165:D210" si="71">((C165&lt;&gt;C164)*1)+((C165=C164)*(H165=H164)*(D164))+((C165=C164)*(H165&lt;&gt;H164)*(D164+1))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E165" s="24">
         <f t="shared" ref="E165:E210" si="72">((H165&lt;&gt;H164)*1)+((H165=H164)*(E164+1))</f>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="F165" s="32" t="str">
         <f t="shared" ref="F165" si="73">_xlfn.CONCAT(C165,".",D165,".",E165)</f>
-        <v>5.5.1</v>
+        <v>5.4.1</v>
       </c>
       <c r="G165" s="19" t="s">
         <v>573</v>
@@ -9720,7 +9720,7 @@
       </c>
       <c r="D166" s="24">
         <f t="shared" si="71"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E166" s="24">
         <f t="shared" si="72"/>
@@ -9728,7 +9728,7 @@
       </c>
       <c r="F166" s="32" t="str">
         <f t="shared" si="40"/>
-        <v>5.5.2</v>
+        <v>5.4.2</v>
       </c>
       <c r="G166" s="19" t="s">
         <v>573</v>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="D167" s="24">
         <f t="shared" si="71"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E167" s="24">
         <f t="shared" si="72"/>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="F167" s="32" t="str">
         <f t="shared" ref="F167:F169" si="74">_xlfn.CONCAT(C167,".",D167,".",E167)</f>
-        <v>5.5.3</v>
+        <v>5.4.3</v>
       </c>
       <c r="G167" s="19" t="s">
         <v>573</v>
@@ -9812,7 +9812,7 @@
       </c>
       <c r="D168" s="24">
         <f t="shared" si="71"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E168" s="24">
         <f t="shared" si="72"/>
@@ -9820,7 +9820,7 @@
       </c>
       <c r="F168" s="32" t="str">
         <f t="shared" si="74"/>
-        <v>5.5.4</v>
+        <v>5.4.4</v>
       </c>
       <c r="G168" s="19" t="s">
         <v>573</v>
@@ -9858,7 +9858,7 @@
       </c>
       <c r="D169" s="24">
         <f t="shared" si="71"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E169" s="24">
         <f t="shared" si="72"/>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="F169" s="32" t="str">
         <f t="shared" si="74"/>
-        <v>5.5.5</v>
+        <v>5.4.5</v>
       </c>
       <c r="G169" s="19" t="s">
         <v>573</v>
@@ -9904,7 +9904,7 @@
       </c>
       <c r="D170" s="24">
         <f t="shared" ref="D170" si="75">((C170&lt;&gt;C169)*1)+((C170=C169)*(H170=H169)*(D169))+((C170=C169)*(H170&lt;&gt;H169)*(D169+1))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E170" s="24">
         <f t="shared" ref="E170" si="76">((H170&lt;&gt;H169)*1)+((H170=H169)*(E169+1))</f>
@@ -9912,7 +9912,7 @@
       </c>
       <c r="F170" s="32" t="str">
         <f t="shared" ref="F170:F239" si="77">_xlfn.CONCAT(C170,".",D170,".",E170)</f>
-        <v>5.6.1</v>
+        <v>5.5.1</v>
       </c>
       <c r="G170" s="19" t="s">
         <v>573</v>
@@ -9950,7 +9950,7 @@
       </c>
       <c r="D171" s="24">
         <f t="shared" si="71"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E171" s="24">
         <f t="shared" si="72"/>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="F171" s="32" t="str">
         <f t="shared" ref="F171:F173" si="78">_xlfn.CONCAT(C171,".",D171,".",E171)</f>
-        <v>5.6.2</v>
+        <v>5.5.2</v>
       </c>
       <c r="G171" s="19" t="s">
         <v>573</v>
@@ -9996,7 +9996,7 @@
       </c>
       <c r="D172" s="24">
         <f t="shared" si="71"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E172" s="24">
         <f t="shared" si="72"/>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="F172" s="32" t="str">
         <f t="shared" si="78"/>
-        <v>5.6.3</v>
+        <v>5.5.3</v>
       </c>
       <c r="G172" s="19" t="s">
         <v>573</v>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="D173" s="24">
         <f t="shared" si="71"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E173" s="24">
         <f t="shared" si="72"/>
@@ -10050,7 +10050,7 @@
       </c>
       <c r="F173" s="32" t="str">
         <f t="shared" si="78"/>
-        <v>5.6.4</v>
+        <v>5.5.4</v>
       </c>
       <c r="G173" s="19" t="s">
         <v>573</v>
@@ -10076,7 +10076,7 @@
       <c r="N173" s="9"/>
       <c r="O173" s="1"/>
     </row>
-    <row r="174" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A174" s="8"/>
       <c r="B174" s="31">
         <f t="shared" si="52"/>
@@ -10122,7 +10122,7 @@
       <c r="N174" s="9"/>
       <c r="O174" s="1"/>
     </row>
-    <row r="175" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A175" s="8"/>
       <c r="B175" s="31">
         <f t="shared" si="52"/>
@@ -10168,7 +10168,7 @@
       <c r="N175" s="9"/>
       <c r="O175" s="1"/>
     </row>
-    <row r="176" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A176" s="8"/>
       <c r="B176" s="31">
         <f t="shared" si="52"/>
@@ -10214,7 +10214,7 @@
       <c r="N176" s="9"/>
       <c r="O176" s="1"/>
     </row>
-    <row r="177" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A177" s="8"/>
       <c r="B177" s="31">
         <f t="shared" si="52"/>
@@ -10260,7 +10260,7 @@
       <c r="N177" s="9"/>
       <c r="O177" s="1"/>
     </row>
-    <row r="178" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A178" s="8"/>
       <c r="B178" s="31">
         <f t="shared" si="52"/>
@@ -10306,7 +10306,7 @@
       <c r="N178" s="9"/>
       <c r="O178" s="1"/>
     </row>
-    <row r="179" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A179" s="8"/>
       <c r="B179" s="31">
         <f t="shared" si="52"/>
@@ -10352,7 +10352,7 @@
       <c r="N179" s="9"/>
       <c r="O179" s="9"/>
     </row>
-    <row r="180" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A180" s="8"/>
       <c r="B180" s="31">
         <f t="shared" si="52"/>
@@ -10398,7 +10398,7 @@
       <c r="N180" s="9"/>
       <c r="O180" s="9"/>
     </row>
-    <row r="181" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A181" s="8"/>
       <c r="B181" s="31">
         <f t="shared" si="52"/>
@@ -10444,7 +10444,7 @@
       <c r="N181" s="9"/>
       <c r="O181" s="9"/>
     </row>
-    <row r="182" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A182" s="8"/>
       <c r="B182" s="31">
         <f t="shared" si="52"/>
@@ -10490,7 +10490,7 @@
       <c r="N182" s="9"/>
       <c r="O182" s="9"/>
     </row>
-    <row r="183" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8"/>
       <c r="B183" s="31">
         <f t="shared" si="52"/>
@@ -10536,7 +10536,7 @@
       <c r="N183" s="9"/>
       <c r="O183" s="9"/>
     </row>
-    <row r="184" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A184" s="8"/>
       <c r="B184" s="31">
         <f t="shared" si="52"/>
@@ -10582,7 +10582,7 @@
       <c r="N184" s="9"/>
       <c r="O184" s="9"/>
     </row>
-    <row r="185" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8"/>
       <c r="B185" s="31">
         <f t="shared" si="52"/>
@@ -10628,7 +10628,7 @@
       <c r="N185" s="9"/>
       <c r="O185" s="9"/>
     </row>
-    <row r="186" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A186" s="8"/>
       <c r="B186" s="31">
         <f t="shared" si="52"/>
@@ -10674,7 +10674,7 @@
       <c r="N186" s="9"/>
       <c r="O186" s="9"/>
     </row>
-    <row r="187" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A187" s="8"/>
       <c r="B187" s="31">
         <f t="shared" si="52"/>
@@ -10720,7 +10720,7 @@
       <c r="N187" s="9"/>
       <c r="O187" s="1"/>
     </row>
-    <row r="188" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A188" s="8"/>
       <c r="B188" s="31">
         <f t="shared" si="52"/>
@@ -10766,7 +10766,7 @@
       <c r="N188" s="9"/>
       <c r="O188" s="1"/>
     </row>
-    <row r="189" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A189" s="8"/>
       <c r="B189" s="31">
         <f t="shared" si="52"/>
@@ -10812,7 +10812,7 @@
       <c r="N189" s="9"/>
       <c r="O189" s="1"/>
     </row>
-    <row r="190" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A190" s="8"/>
       <c r="B190" s="31">
         <f t="shared" si="52"/>
@@ -10858,7 +10858,7 @@
       <c r="N190" s="9"/>
       <c r="O190" s="1"/>
     </row>
-    <row r="191" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A191" s="8"/>
       <c r="B191" s="31">
         <f t="shared" si="52"/>
@@ -10904,7 +10904,7 @@
       <c r="N191" s="9"/>
       <c r="O191" s="1"/>
     </row>
-    <row r="192" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A192" s="8"/>
       <c r="B192" s="31">
         <f t="shared" si="52"/>
@@ -10950,7 +10950,7 @@
       <c r="N192" s="9"/>
       <c r="O192" s="1"/>
     </row>
-    <row r="193" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A193" s="8"/>
       <c r="B193" s="31">
         <f t="shared" si="52"/>
@@ -10996,7 +10996,7 @@
       <c r="N193" s="9"/>
       <c r="O193" s="1"/>
     </row>
-    <row r="194" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A194" s="8"/>
       <c r="B194" s="31">
         <f t="shared" si="52"/>
@@ -11042,7 +11042,7 @@
       <c r="N194" s="9"/>
       <c r="O194" s="1"/>
     </row>
-    <row r="195" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A195" s="8"/>
       <c r="B195" s="31">
         <f t="shared" si="52"/>
@@ -11088,7 +11088,7 @@
       <c r="N195" s="9"/>
       <c r="O195" s="1"/>
     </row>
-    <row r="196" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A196" s="8"/>
       <c r="B196" s="31">
         <f t="shared" si="52"/>
@@ -11134,7 +11134,7 @@
       <c r="N196" s="9"/>
       <c r="O196" s="1"/>
     </row>
-    <row r="197" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A197" s="8"/>
       <c r="B197" s="31">
         <f t="shared" si="52"/>
@@ -11180,7 +11180,7 @@
       <c r="N197" s="9"/>
       <c r="O197" s="1"/>
     </row>
-    <row r="198" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A198" s="8"/>
       <c r="B198" s="31">
         <f t="shared" si="52"/>
@@ -11226,7 +11226,7 @@
       <c r="N198" s="9"/>
       <c r="O198" s="1"/>
     </row>
-    <row r="199" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A199" s="8"/>
       <c r="B199" s="31">
         <f t="shared" si="52"/>
@@ -11272,7 +11272,7 @@
       <c r="N199" s="9"/>
       <c r="O199" s="1"/>
     </row>
-    <row r="200" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A200" s="8"/>
       <c r="B200" s="31">
         <f t="shared" si="52"/>
@@ -11318,7 +11318,7 @@
       <c r="N200" s="9"/>
       <c r="O200" s="1"/>
     </row>
-    <row r="201" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A201" s="8"/>
       <c r="B201" s="31">
         <f t="shared" ref="B201:B264" si="87">+B200+1</f>
@@ -11364,7 +11364,7 @@
       <c r="N201" s="9"/>
       <c r="O201" s="1"/>
     </row>
-    <row r="202" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A202" s="8"/>
       <c r="B202" s="31">
         <f t="shared" si="87"/>
@@ -11410,7 +11410,7 @@
       <c r="N202" s="9"/>
       <c r="O202" s="1"/>
     </row>
-    <row r="203" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A203" s="1"/>
       <c r="B203" s="31">
         <f t="shared" si="87"/>
@@ -11456,7 +11456,7 @@
       <c r="N203" s="9"/>
       <c r="O203" s="1"/>
     </row>
-    <row r="204" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A204" s="1"/>
       <c r="B204" s="31">
         <f t="shared" si="87"/>
@@ -11502,7 +11502,7 @@
       <c r="N204" s="9"/>
       <c r="O204" s="1"/>
     </row>
-    <row r="205" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A205" s="1"/>
       <c r="B205" s="31">
         <f t="shared" si="87"/>
@@ -11548,7 +11548,7 @@
       <c r="N205" s="9"/>
       <c r="O205" s="1"/>
     </row>
-    <row r="206" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A206" s="1"/>
       <c r="B206" s="31">
         <f t="shared" si="87"/>
@@ -11594,7 +11594,7 @@
       <c r="N206" s="9"/>
       <c r="O206" s="1"/>
     </row>
-    <row r="207" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A207" s="1"/>
       <c r="B207" s="31">
         <f t="shared" si="87"/>
@@ -11640,7 +11640,7 @@
       <c r="N207" s="9"/>
       <c r="O207" s="1"/>
     </row>
-    <row r="208" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A208" s="1"/>
       <c r="B208" s="31">
         <f t="shared" si="87"/>
@@ -11686,7 +11686,7 @@
       <c r="N208" s="9"/>
       <c r="O208" s="1"/>
     </row>
-    <row r="209" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A209" s="1"/>
       <c r="B209" s="31">
         <f t="shared" si="87"/>
@@ -11732,7 +11732,7 @@
       <c r="N209" s="9"/>
       <c r="O209" s="1"/>
     </row>
-    <row r="210" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A210" s="1"/>
       <c r="B210" s="31">
         <f t="shared" si="87"/>
@@ -11778,7 +11778,7 @@
       <c r="N210" s="9"/>
       <c r="O210" s="1"/>
     </row>
-    <row r="211" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A211" s="1"/>
       <c r="B211" s="31">
         <f t="shared" si="87"/>
@@ -11824,7 +11824,7 @@
       <c r="N211" s="9"/>
       <c r="O211" s="1"/>
     </row>
-    <row r="212" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A212" s="8"/>
       <c r="B212" s="31">
         <f t="shared" si="87"/>
@@ -11870,7 +11870,7 @@
       <c r="N212" s="9"/>
       <c r="O212" s="9"/>
     </row>
-    <row r="213" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A213" s="8"/>
       <c r="B213" s="31">
         <f t="shared" si="87"/>
@@ -11916,7 +11916,7 @@
       <c r="N213" s="9"/>
       <c r="O213" s="9"/>
     </row>
-    <row r="214" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A214" s="8"/>
       <c r="B214" s="31">
         <f t="shared" si="87"/>
@@ -11962,7 +11962,7 @@
       <c r="N214" s="9"/>
       <c r="O214" s="9"/>
     </row>
-    <row r="215" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A215" s="8"/>
       <c r="B215" s="31">
         <f t="shared" si="87"/>
@@ -12008,7 +12008,7 @@
       <c r="N215" s="9"/>
       <c r="O215" s="9"/>
     </row>
-    <row r="216" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A216" s="8"/>
       <c r="B216" s="31">
         <f t="shared" si="87"/>
@@ -12054,7 +12054,7 @@
       <c r="N216" s="9"/>
       <c r="O216" s="9"/>
     </row>
-    <row r="217" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A217" s="8"/>
       <c r="B217" s="31">
         <f t="shared" si="87"/>
@@ -12100,7 +12100,7 @@
       <c r="N217" s="9"/>
       <c r="O217" s="9"/>
     </row>
-    <row r="218" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A218" s="8"/>
       <c r="B218" s="31">
         <f t="shared" si="87"/>
@@ -12146,7 +12146,7 @@
       <c r="N218" s="9"/>
       <c r="O218" s="9"/>
     </row>
-    <row r="219" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A219" s="8"/>
       <c r="B219" s="31">
         <f t="shared" si="87"/>
@@ -12192,7 +12192,7 @@
       <c r="N219" s="9"/>
       <c r="O219" s="9"/>
     </row>
-    <row r="220" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A220" s="8"/>
       <c r="B220" s="31">
         <f t="shared" si="87"/>
@@ -12238,7 +12238,7 @@
       <c r="N220" s="9"/>
       <c r="O220" s="9"/>
     </row>
-    <row r="221" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A221" s="1"/>
       <c r="B221" s="31">
         <f t="shared" si="87"/>
@@ -12284,7 +12284,7 @@
       <c r="N221" s="9"/>
       <c r="O221" s="1"/>
     </row>
-    <row r="222" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A222" s="1"/>
       <c r="B222" s="31">
         <f t="shared" si="87"/>
@@ -12330,7 +12330,7 @@
       <c r="N222" s="9"/>
       <c r="O222" s="1"/>
     </row>
-    <row r="223" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A223" s="1"/>
       <c r="B223" s="31">
         <f t="shared" si="87"/>
@@ -12376,7 +12376,7 @@
       <c r="N223" s="9"/>
       <c r="O223" s="1"/>
     </row>
-    <row r="224" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A224" s="1"/>
       <c r="B224" s="31">
         <f t="shared" si="87"/>
@@ -12422,7 +12422,7 @@
       <c r="N224" s="9"/>
       <c r="O224" s="1"/>
     </row>
-    <row r="225" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A225" s="1"/>
       <c r="B225" s="31">
         <f t="shared" si="87"/>
@@ -12468,7 +12468,7 @@
       <c r="N225" s="9"/>
       <c r="O225" s="1"/>
     </row>
-    <row r="226" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A226" s="1"/>
       <c r="B226" s="31">
         <f t="shared" si="87"/>
@@ -12514,7 +12514,7 @@
       <c r="N226" s="9"/>
       <c r="O226" s="1"/>
     </row>
-    <row r="227" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A227" s="1"/>
       <c r="B227" s="31">
         <f t="shared" si="87"/>
@@ -12560,7 +12560,7 @@
       <c r="N227" s="9"/>
       <c r="O227" s="1"/>
     </row>
-    <row r="228" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A228" s="1"/>
       <c r="B228" s="31">
         <f t="shared" si="87"/>
@@ -12606,7 +12606,7 @@
       <c r="N228" s="9"/>
       <c r="O228" s="1"/>
     </row>
-    <row r="229" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A229" s="1"/>
       <c r="B229" s="31">
         <f t="shared" si="87"/>
@@ -12652,7 +12652,7 @@
       <c r="N229" s="9"/>
       <c r="O229" s="1"/>
     </row>
-    <row r="230" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A230" s="1"/>
       <c r="B230" s="31">
         <f t="shared" si="87"/>
@@ -12698,7 +12698,7 @@
       <c r="N230" s="9"/>
       <c r="O230" s="1"/>
     </row>
-    <row r="231" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A231" s="1"/>
       <c r="B231" s="31">
         <f t="shared" si="87"/>
@@ -12744,7 +12744,7 @@
       <c r="N231" s="9"/>
       <c r="O231" s="1"/>
     </row>
-    <row r="232" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A232" s="1"/>
       <c r="B232" s="31">
         <f t="shared" si="87"/>
@@ -12790,7 +12790,7 @@
       <c r="N232" s="9"/>
       <c r="O232" s="1"/>
     </row>
-    <row r="233" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A233" s="1"/>
       <c r="B233" s="31">
         <f t="shared" si="87"/>
@@ -12836,7 +12836,7 @@
       <c r="N233" s="9"/>
       <c r="O233" s="1"/>
     </row>
-    <row r="234" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A234" s="1"/>
       <c r="B234" s="31">
         <f t="shared" si="87"/>
@@ -12882,7 +12882,7 @@
       <c r="N234" s="9"/>
       <c r="O234" s="1"/>
     </row>
-    <row r="235" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A235" s="1"/>
       <c r="B235" s="31">
         <f t="shared" si="87"/>
@@ -12928,7 +12928,7 @@
       <c r="N235" s="9"/>
       <c r="O235" s="1"/>
     </row>
-    <row r="236" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A236" s="1"/>
       <c r="B236" s="31">
         <f t="shared" si="87"/>
@@ -12974,7 +12974,7 @@
       <c r="N236" s="9"/>
       <c r="O236" s="1"/>
     </row>
-    <row r="237" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A237" s="1"/>
       <c r="B237" s="31">
         <f t="shared" si="87"/>
@@ -13020,7 +13020,7 @@
       <c r="N237" s="9"/>
       <c r="O237" s="1"/>
     </row>
-    <row r="238" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A238" s="1"/>
       <c r="B238" s="31">
         <f t="shared" si="87"/>
@@ -13066,7 +13066,7 @@
       <c r="N238" s="9"/>
       <c r="O238" s="1"/>
     </row>
-    <row r="239" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A239" s="1"/>
       <c r="B239" s="31">
         <f t="shared" si="87"/>
@@ -13112,7 +13112,7 @@
       <c r="N239" s="9"/>
       <c r="O239" s="1"/>
     </row>
-    <row r="240" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A240" s="1"/>
       <c r="B240" s="31">
         <f t="shared" si="87"/>
@@ -13158,7 +13158,7 @@
       <c r="N240" s="9"/>
       <c r="O240" s="1"/>
     </row>
-    <row r="241" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A241" s="1"/>
       <c r="B241" s="31">
         <f t="shared" si="87"/>
@@ -13204,7 +13204,7 @@
       <c r="N241" s="9"/>
       <c r="O241" s="1"/>
     </row>
-    <row r="242" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A242" s="8"/>
       <c r="B242" s="31">
         <f t="shared" si="87"/>
@@ -13250,7 +13250,7 @@
       <c r="N242" s="9"/>
       <c r="O242" s="9"/>
     </row>
-    <row r="243" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A243" s="8"/>
       <c r="B243" s="31">
         <f t="shared" si="87"/>
@@ -13296,7 +13296,7 @@
       <c r="N243" s="9"/>
       <c r="O243" s="9"/>
     </row>
-    <row r="244" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A244" s="8"/>
       <c r="B244" s="31">
         <f t="shared" si="87"/>
@@ -13342,7 +13342,7 @@
       <c r="N244" s="9"/>
       <c r="O244" s="9"/>
     </row>
-    <row r="245" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A245" s="8"/>
       <c r="B245" s="31">
         <f t="shared" si="87"/>
@@ -13388,7 +13388,7 @@
       <c r="N245" s="9"/>
       <c r="O245" s="9"/>
     </row>
-    <row r="246" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A246" s="8"/>
       <c r="B246" s="31">
         <f t="shared" si="87"/>
@@ -13434,7 +13434,7 @@
       <c r="N246" s="9"/>
       <c r="O246" s="9"/>
     </row>
-    <row r="247" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A247" s="8"/>
       <c r="B247" s="31">
         <f t="shared" si="87"/>
@@ -13480,7 +13480,7 @@
       <c r="N247" s="9"/>
       <c r="O247" s="9"/>
     </row>
-    <row r="248" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A248" s="8"/>
       <c r="B248" s="31">
         <f t="shared" si="87"/>
@@ -13526,7 +13526,7 @@
       <c r="N248" s="9"/>
       <c r="O248" s="9"/>
     </row>
-    <row r="249" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A249" s="8"/>
       <c r="B249" s="31">
         <f t="shared" si="87"/>
@@ -13572,7 +13572,7 @@
       <c r="N249" s="9"/>
       <c r="O249" s="9"/>
     </row>
-    <row r="250" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A250" s="8"/>
       <c r="B250" s="31">
         <f t="shared" si="87"/>
@@ -13618,7 +13618,7 @@
       <c r="N250" s="9"/>
       <c r="O250" s="9"/>
     </row>
-    <row r="251" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A251" s="1"/>
       <c r="B251" s="31">
         <f t="shared" si="87"/>
@@ -13664,7 +13664,7 @@
       <c r="N251" s="9"/>
       <c r="O251" s="1"/>
     </row>
-    <row r="252" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A252" s="1"/>
       <c r="B252" s="31">
         <f t="shared" si="87"/>
@@ -13710,7 +13710,7 @@
       <c r="N252" s="9"/>
       <c r="O252" s="1"/>
     </row>
-    <row r="253" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A253" s="1"/>
       <c r="B253" s="31">
         <f t="shared" si="87"/>
@@ -13756,7 +13756,7 @@
       <c r="N253" s="9"/>
       <c r="O253" s="1"/>
     </row>
-    <row r="254" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A254" s="1"/>
       <c r="B254" s="31">
         <f t="shared" si="87"/>
@@ -13802,7 +13802,7 @@
       <c r="N254" s="9"/>
       <c r="O254" s="1"/>
     </row>
-    <row r="255" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A255" s="1"/>
       <c r="B255" s="31">
         <f t="shared" si="87"/>
@@ -13848,7 +13848,7 @@
       <c r="N255" s="9"/>
       <c r="O255" s="1"/>
     </row>
-    <row r="256" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A256" s="1"/>
       <c r="B256" s="31">
         <f t="shared" si="87"/>
@@ -13894,7 +13894,7 @@
       <c r="N256" s="9"/>
       <c r="O256" s="1"/>
     </row>
-    <row r="257" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A257" s="1"/>
       <c r="B257" s="31">
         <f t="shared" si="87"/>
@@ -13940,7 +13940,7 @@
       <c r="N257" s="9"/>
       <c r="O257" s="1"/>
     </row>
-    <row r="258" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A258" s="1"/>
       <c r="B258" s="31">
         <f t="shared" si="87"/>
@@ -13986,7 +13986,7 @@
       <c r="N258" s="9"/>
       <c r="O258" s="1"/>
     </row>
-    <row r="259" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A259" s="1"/>
       <c r="B259" s="31">
         <f t="shared" si="87"/>
@@ -14032,7 +14032,7 @@
       <c r="N259" s="9"/>
       <c r="O259" s="1"/>
     </row>
-    <row r="260" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A260" s="1"/>
       <c r="B260" s="31">
         <f t="shared" si="87"/>
@@ -14078,7 +14078,7 @@
       <c r="N260" s="9"/>
       <c r="O260" s="1"/>
     </row>
-    <row r="261" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A261" s="1"/>
       <c r="B261" s="31">
         <f t="shared" si="87"/>
@@ -14124,7 +14124,7 @@
       <c r="N261" s="9"/>
       <c r="O261" s="1"/>
     </row>
-    <row r="262" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A262" s="1"/>
       <c r="B262" s="31">
         <f t="shared" si="87"/>
@@ -14170,7 +14170,7 @@
       <c r="N262" s="9"/>
       <c r="O262" s="1"/>
     </row>
-    <row r="263" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A263" s="1"/>
       <c r="B263" s="31">
         <f t="shared" si="87"/>
@@ -14216,7 +14216,7 @@
       <c r="N263" s="9"/>
       <c r="O263" s="1"/>
     </row>
-    <row r="264" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A264" s="1"/>
       <c r="B264" s="31">
         <f t="shared" si="87"/>
@@ -14262,7 +14262,7 @@
       <c r="N264" s="9"/>
       <c r="O264" s="1"/>
     </row>
-    <row r="265" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A265" s="1"/>
       <c r="B265" s="31">
         <f t="shared" ref="B265:B293" si="119">+B264+1</f>
@@ -14308,7 +14308,7 @@
       <c r="N265" s="9"/>
       <c r="O265" s="1"/>
     </row>
-    <row r="266" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A266" s="1"/>
       <c r="B266" s="31">
         <f t="shared" si="119"/>
@@ -14354,7 +14354,7 @@
       <c r="N266" s="9"/>
       <c r="O266" s="1"/>
     </row>
-    <row r="267" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A267" s="1"/>
       <c r="B267" s="31">
         <f t="shared" si="119"/>
@@ -14400,7 +14400,7 @@
       <c r="N267" s="9"/>
       <c r="O267" s="1"/>
     </row>
-    <row r="268" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A268" s="1"/>
       <c r="B268" s="31">
         <f t="shared" si="119"/>
@@ -14446,7 +14446,7 @@
       <c r="N268" s="9"/>
       <c r="O268" s="1"/>
     </row>
-    <row r="269" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A269" s="1"/>
       <c r="B269" s="31">
         <f t="shared" si="119"/>
@@ -14492,7 +14492,7 @@
       <c r="N269" s="9"/>
       <c r="O269" s="1"/>
     </row>
-    <row r="270" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A270" s="1"/>
       <c r="B270" s="31">
         <f t="shared" si="119"/>
@@ -14538,7 +14538,7 @@
       <c r="N270" s="9"/>
       <c r="O270" s="1"/>
     </row>
-    <row r="271" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A271" s="1"/>
       <c r="B271" s="31">
         <f t="shared" si="119"/>
@@ -14584,7 +14584,7 @@
       <c r="N271" s="9"/>
       <c r="O271" s="1"/>
     </row>
-    <row r="272" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A272" s="1"/>
       <c r="B272" s="31">
         <f t="shared" si="119"/>
@@ -14630,7 +14630,7 @@
       <c r="N272" s="9"/>
       <c r="O272" s="1"/>
     </row>
-    <row r="273" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A273" s="1"/>
       <c r="B273" s="31">
         <f t="shared" si="119"/>
@@ -14676,7 +14676,7 @@
       <c r="N273" s="9"/>
       <c r="O273" s="1"/>
     </row>
-    <row r="274" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A274" s="1"/>
       <c r="B274" s="31">
         <f t="shared" si="119"/>
@@ -14722,7 +14722,7 @@
       <c r="N274" s="9"/>
       <c r="O274" s="1"/>
     </row>
-    <row r="275" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A275" s="1"/>
       <c r="B275" s="31">
         <f t="shared" si="119"/>
@@ -14768,7 +14768,7 @@
       <c r="N275" s="9"/>
       <c r="O275" s="1"/>
     </row>
-    <row r="276" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A276" s="1"/>
       <c r="B276" s="31">
         <f t="shared" si="119"/>
@@ -14814,7 +14814,7 @@
       <c r="N276" s="9"/>
       <c r="O276" s="1"/>
     </row>
-    <row r="277" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A277" s="1"/>
       <c r="B277" s="31">
         <f t="shared" si="119"/>
@@ -14860,7 +14860,7 @@
       <c r="N277" s="9"/>
       <c r="O277" s="1"/>
     </row>
-    <row r="278" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A278" s="1"/>
       <c r="B278" s="31">
         <f t="shared" si="119"/>
@@ -14906,7 +14906,7 @@
       <c r="N278" s="9"/>
       <c r="O278" s="1"/>
     </row>
-    <row r="279" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A279" s="1"/>
       <c r="B279" s="31">
         <f t="shared" si="119"/>
@@ -14952,7 +14952,7 @@
       <c r="N279" s="9"/>
       <c r="O279" s="1"/>
     </row>
-    <row r="280" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A280" s="1"/>
       <c r="B280" s="31">
         <f t="shared" si="119"/>
@@ -14998,7 +14998,7 @@
       <c r="N280" s="9"/>
       <c r="O280" s="1"/>
     </row>
-    <row r="281" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A281" s="1"/>
       <c r="B281" s="31">
         <f t="shared" si="119"/>
@@ -15044,7 +15044,7 @@
       <c r="N281" s="9"/>
       <c r="O281" s="1"/>
     </row>
-    <row r="282" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A282" s="1"/>
       <c r="B282" s="31">
         <f t="shared" si="119"/>
@@ -15090,7 +15090,7 @@
       <c r="N282" s="9"/>
       <c r="O282" s="1"/>
     </row>
-    <row r="283" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A283" s="1"/>
       <c r="B283" s="31">
         <f t="shared" si="119"/>
@@ -15136,7 +15136,7 @@
       <c r="N283" s="9"/>
       <c r="O283" s="1"/>
     </row>
-    <row r="284" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A284" s="1"/>
       <c r="B284" s="31">
         <f t="shared" si="119"/>
@@ -15182,7 +15182,7 @@
       <c r="N284" s="9"/>
       <c r="O284" s="1"/>
     </row>
-    <row r="285" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A285" s="1"/>
       <c r="B285" s="31">
         <f t="shared" si="119"/>
@@ -15228,7 +15228,7 @@
       <c r="N285" s="9"/>
       <c r="O285" s="1"/>
     </row>
-    <row r="286" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A286" s="1"/>
       <c r="B286" s="31">
         <f t="shared" si="119"/>
@@ -15274,7 +15274,7 @@
       <c r="N286" s="9"/>
       <c r="O286" s="1"/>
     </row>
-    <row r="287" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A287" s="1"/>
       <c r="B287" s="31">
         <f t="shared" si="119"/>
@@ -15296,7 +15296,7 @@
         <f t="shared" si="101"/>
         <v>13.1.1</v>
       </c>
-      <c r="G287" s="10" t="s">
+      <c r="G287" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H287" s="19" t="s">
@@ -15320,7 +15320,7 @@
       <c r="N287" s="9"/>
       <c r="O287" s="1"/>
     </row>
-    <row r="288" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A288" s="1"/>
       <c r="B288" s="31">
         <f t="shared" si="119"/>
@@ -15342,7 +15342,7 @@
         <f t="shared" si="101"/>
         <v>13.2.1</v>
       </c>
-      <c r="G288" s="10" t="s">
+      <c r="G288" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H288" s="19" t="s">
@@ -15366,7 +15366,7 @@
       <c r="N288" s="9"/>
       <c r="O288" s="1"/>
     </row>
-    <row r="289" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A289" s="1"/>
       <c r="B289" s="31">
         <f t="shared" si="119"/>
@@ -15388,7 +15388,7 @@
         <f t="shared" si="101"/>
         <v>13.3.1</v>
       </c>
-      <c r="G289" s="10" t="s">
+      <c r="G289" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H289" s="19" t="s">
@@ -15412,7 +15412,7 @@
       <c r="N289" s="9"/>
       <c r="O289" s="1"/>
     </row>
-    <row r="290" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A290" s="1"/>
       <c r="B290" s="31">
         <f t="shared" si="119"/>
@@ -15458,7 +15458,7 @@
       <c r="N290" s="9"/>
       <c r="O290" s="1"/>
     </row>
-    <row r="291" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A291" s="1"/>
       <c r="B291" s="31">
         <f t="shared" si="119"/>
@@ -15504,7 +15504,7 @@
       <c r="N291" s="9"/>
       <c r="O291" s="1"/>
     </row>
-    <row r="292" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A292" s="1"/>
       <c r="B292" s="31">
         <f t="shared" si="119"/>
@@ -15550,7 +15550,7 @@
       <c r="N292" s="9"/>
       <c r="O292" s="1"/>
     </row>
-    <row r="293" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A293" s="1"/>
       <c r="B293" s="31">
         <f t="shared" si="119"/>
@@ -15596,7 +15596,7 @@
       <c r="N293" s="9"/>
       <c r="O293" s="1"/>
     </row>
-    <row r="294" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A294" s="1"/>
       <c r="B294" s="31">
         <f t="shared" ref="B294:B295" si="126">+B293+1</f>
@@ -15642,7 +15642,7 @@
       <c r="N294" s="9"/>
       <c r="O294" s="1"/>
     </row>
-    <row r="295" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A295" s="1"/>
       <c r="B295" s="31">
         <f t="shared" si="126"/>
@@ -15688,7 +15688,7 @@
       <c r="N295" s="9"/>
       <c r="O295" s="1"/>
     </row>
-    <row r="296" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A296" s="1"/>
       <c r="B296" s="31">
         <f t="shared" ref="B296:B359" si="130">+B295+1</f>
@@ -15734,7 +15734,7 @@
       <c r="N296" s="9"/>
       <c r="O296" s="1"/>
     </row>
-    <row r="297" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" s="8"/>
       <c r="B297" s="31">
         <f t="shared" si="130"/>
@@ -15780,7 +15780,7 @@
       <c r="N297" s="1"/>
       <c r="O297" s="1"/>
     </row>
-    <row r="298" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" s="8"/>
       <c r="B298" s="31">
         <f t="shared" si="130"/>
@@ -15825,7 +15825,7 @@
       <c r="N298" s="1"/>
       <c r="O298" s="1"/>
     </row>
-    <row r="299" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" s="8"/>
       <c r="B299" s="31">
         <f t="shared" si="130"/>
@@ -15870,7 +15870,7 @@
       <c r="N299" s="1"/>
       <c r="O299" s="1"/>
     </row>
-    <row r="300" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" s="8"/>
       <c r="B300" s="31">
         <f t="shared" si="130"/>
@@ -15915,7 +15915,7 @@
       <c r="N300" s="1"/>
       <c r="O300" s="1"/>
     </row>
-    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="7"/>
       <c r="B301" s="31">
         <f t="shared" si="130"/>
@@ -15960,7 +15960,7 @@
       <c r="N301" s="7"/>
       <c r="O301" s="7"/>
     </row>
-    <row r="302" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="7"/>
       <c r="B302" s="31">
         <f t="shared" si="130"/>
@@ -16005,7 +16005,7 @@
       <c r="N302" s="7"/>
       <c r="O302" s="7"/>
     </row>
-    <row r="303" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="7"/>
       <c r="B303" s="31">
         <f t="shared" si="130"/>
@@ -16050,7 +16050,7 @@
       <c r="N303" s="7"/>
       <c r="O303" s="7"/>
     </row>
-    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="7"/>
       <c r="B304" s="31">
         <f t="shared" si="130"/>
@@ -16095,7 +16095,7 @@
       <c r="N304" s="7"/>
       <c r="O304" s="7"/>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="7"/>
       <c r="B305" s="31">
         <f t="shared" si="130"/>
@@ -16140,7 +16140,7 @@
       <c r="N305" s="7"/>
       <c r="O305" s="7"/>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="7"/>
       <c r="B306" s="31">
         <f t="shared" si="130"/>
@@ -16185,7 +16185,7 @@
       <c r="N306" s="7"/>
       <c r="O306" s="7"/>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="7"/>
       <c r="B307" s="31">
         <f t="shared" si="130"/>
@@ -16230,7 +16230,7 @@
       <c r="N307" s="7"/>
       <c r="O307" s="7"/>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="7"/>
       <c r="B308" s="31">
         <f t="shared" si="130"/>
@@ -16275,7 +16275,7 @@
       <c r="N308" s="7"/>
       <c r="O308" s="7"/>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="7"/>
       <c r="B309" s="31">
         <f t="shared" si="130"/>
@@ -16320,7 +16320,7 @@
       <c r="N309" s="7"/>
       <c r="O309" s="7"/>
     </row>
-    <row r="310" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" s="1"/>
       <c r="B310" s="31">
         <f t="shared" si="130"/>
@@ -16365,7 +16365,7 @@
       <c r="N310" s="1"/>
       <c r="O310" s="1"/>
     </row>
-    <row r="311" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" s="1"/>
       <c r="B311" s="31">
         <f t="shared" si="130"/>
@@ -16410,7 +16410,7 @@
       <c r="N311" s="1"/>
       <c r="O311" s="1"/>
     </row>
-    <row r="312" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" s="1"/>
       <c r="B312" s="31">
         <f t="shared" si="130"/>
@@ -16455,7 +16455,7 @@
       <c r="N312" s="1"/>
       <c r="O312" s="1"/>
     </row>
-    <row r="313" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" s="1"/>
       <c r="B313" s="31">
         <f t="shared" si="130"/>
@@ -16500,7 +16500,7 @@
       <c r="N313" s="1"/>
       <c r="O313" s="1"/>
     </row>
-    <row r="314" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" s="1"/>
       <c r="B314" s="31">
         <f t="shared" si="130"/>
@@ -16815,7 +16815,7 @@
       <c r="N320" s="1"/>
       <c r="O320" s="1"/>
     </row>
-    <row r="321" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" s="1"/>
       <c r="B321" s="31">
         <f t="shared" si="130"/>
@@ -16860,7 +16860,7 @@
       <c r="N321" s="1"/>
       <c r="O321" s="1"/>
     </row>
-    <row r="322" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" s="1"/>
       <c r="B322" s="31">
         <f t="shared" si="130"/>
@@ -16905,7 +16905,7 @@
       <c r="N322" s="1"/>
       <c r="O322" s="1"/>
     </row>
-    <row r="323" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" s="1"/>
       <c r="B323" s="31">
         <f t="shared" si="130"/>
@@ -16950,7 +16950,7 @@
       <c r="N323" s="1"/>
       <c r="O323" s="1"/>
     </row>
-    <row r="324" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" s="1"/>
       <c r="B324" s="31">
         <f t="shared" si="130"/>
@@ -16995,7 +16995,7 @@
       <c r="N324" s="1"/>
       <c r="O324" s="1"/>
     </row>
-    <row r="325" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" s="1"/>
       <c r="B325" s="31">
         <f t="shared" si="130"/>
@@ -17040,7 +17040,7 @@
       <c r="N325" s="1"/>
       <c r="O325" s="1"/>
     </row>
-    <row r="326" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" s="1"/>
       <c r="B326" s="31">
         <f t="shared" si="130"/>
@@ -17085,7 +17085,7 @@
       <c r="N326" s="1"/>
       <c r="O326" s="1"/>
     </row>
-    <row r="327" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" s="1"/>
       <c r="B327" s="31">
         <f t="shared" si="130"/>
@@ -17130,7 +17130,7 @@
       <c r="N327" s="1"/>
       <c r="O327" s="1"/>
     </row>
-    <row r="328" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" s="1"/>
       <c r="B328" s="31">
         <f t="shared" si="130"/>
@@ -17175,7 +17175,7 @@
       <c r="N328" s="1"/>
       <c r="O328" s="1"/>
     </row>
-    <row r="329" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" s="1"/>
       <c r="B329" s="31">
         <f t="shared" si="130"/>
@@ -17220,7 +17220,7 @@
       <c r="N329" s="1"/>
       <c r="O329" s="1"/>
     </row>
-    <row r="330" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" s="1"/>
       <c r="B330" s="31">
         <f t="shared" si="130"/>
@@ -17265,7 +17265,7 @@
       <c r="N330" s="1"/>
       <c r="O330" s="1"/>
     </row>
-    <row r="331" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" s="1"/>
       <c r="B331" s="31">
         <f t="shared" si="130"/>
@@ -17310,7 +17310,7 @@
       <c r="N331" s="1"/>
       <c r="O331" s="1"/>
     </row>
-    <row r="332" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" s="1"/>
       <c r="B332" s="31">
         <f t="shared" si="130"/>
@@ -17355,7 +17355,7 @@
       <c r="N332" s="1"/>
       <c r="O332" s="1"/>
     </row>
-    <row r="333" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" s="1"/>
       <c r="B333" s="31">
         <f t="shared" si="130"/>
@@ -17400,7 +17400,7 @@
       <c r="N333" s="1"/>
       <c r="O333" s="1"/>
     </row>
-    <row r="334" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" s="1"/>
       <c r="B334" s="31">
         <f t="shared" si="130"/>
@@ -17445,7 +17445,7 @@
       <c r="N334" s="1"/>
       <c r="O334" s="1"/>
     </row>
-    <row r="335" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" s="1"/>
       <c r="B335" s="31">
         <f t="shared" si="130"/>
@@ -17490,7 +17490,7 @@
       <c r="N335" s="1"/>
       <c r="O335" s="1"/>
     </row>
-    <row r="336" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" s="1"/>
       <c r="B336" s="31">
         <f t="shared" si="130"/>
@@ -17535,7 +17535,7 @@
       <c r="N336" s="1"/>
       <c r="O336" s="1"/>
     </row>
-    <row r="337" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" s="1"/>
       <c r="B337" s="31">
         <f t="shared" si="130"/>
@@ -17580,7 +17580,7 @@
       <c r="N337" s="1"/>
       <c r="O337" s="1"/>
     </row>
-    <row r="338" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" s="1"/>
       <c r="B338" s="31">
         <f t="shared" si="130"/>
@@ -17625,7 +17625,7 @@
       <c r="N338" s="1"/>
       <c r="O338" s="1"/>
     </row>
-    <row r="339" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" s="1"/>
       <c r="B339" s="31">
         <f t="shared" si="130"/>
@@ -17670,7 +17670,7 @@
       <c r="N339" s="1"/>
       <c r="O339" s="1"/>
     </row>
-    <row r="340" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" s="1"/>
       <c r="B340" s="31">
         <f t="shared" si="130"/>
@@ -17715,7 +17715,7 @@
       <c r="N340" s="1"/>
       <c r="O340" s="1"/>
     </row>
-    <row r="341" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" s="1"/>
       <c r="B341" s="31">
         <f t="shared" si="130"/>
@@ -17760,7 +17760,7 @@
       <c r="N341" s="1"/>
       <c r="O341" s="1"/>
     </row>
-    <row r="342" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" s="1"/>
       <c r="B342" s="31">
         <f t="shared" si="130"/>
@@ -17805,7 +17805,7 @@
       <c r="N342" s="1"/>
       <c r="O342" s="1"/>
     </row>
-    <row r="343" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" s="1"/>
       <c r="B343" s="31">
         <f t="shared" si="130"/>
@@ -17850,7 +17850,7 @@
       <c r="N343" s="1"/>
       <c r="O343" s="1"/>
     </row>
-    <row r="344" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" s="1"/>
       <c r="B344" s="31">
         <f t="shared" si="130"/>
@@ -17895,7 +17895,7 @@
       <c r="N344" s="1"/>
       <c r="O344" s="1"/>
     </row>
-    <row r="345" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" s="1"/>
       <c r="B345" s="31">
         <f t="shared" si="130"/>
@@ -17940,7 +17940,7 @@
       <c r="N345" s="1"/>
       <c r="O345" s="1"/>
     </row>
-    <row r="346" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" s="1"/>
       <c r="B346" s="31">
         <f t="shared" si="130"/>
@@ -17985,7 +17985,7 @@
       <c r="N346" s="1"/>
       <c r="O346" s="1"/>
     </row>
-    <row r="347" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" s="1"/>
       <c r="B347" s="31">
         <f t="shared" si="130"/>
@@ -18030,7 +18030,7 @@
       <c r="N347" s="1"/>
       <c r="O347" s="1"/>
     </row>
-    <row r="348" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" s="1"/>
       <c r="B348" s="31">
         <f t="shared" si="130"/>
@@ -18075,7 +18075,7 @@
       <c r="N348" s="1"/>
       <c r="O348" s="1"/>
     </row>
-    <row r="349" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" s="1"/>
       <c r="B349" s="31">
         <f t="shared" si="130"/>
@@ -18096,7 +18096,7 @@
         <f t="shared" si="129"/>
         <v>13.1.0</v>
       </c>
-      <c r="G349" s="10" t="s">
+      <c r="G349" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H349" s="19" t="s">
@@ -18120,7 +18120,7 @@
       <c r="N349" s="1"/>
       <c r="O349" s="1"/>
     </row>
-    <row r="350" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" s="1"/>
       <c r="B350" s="31">
         <f t="shared" si="130"/>
@@ -18141,7 +18141,7 @@
         <f t="shared" si="129"/>
         <v>13.2.0</v>
       </c>
-      <c r="G350" s="10" t="s">
+      <c r="G350" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H350" s="19" t="s">
@@ -18165,7 +18165,7 @@
       <c r="N350" s="1"/>
       <c r="O350" s="1"/>
     </row>
-    <row r="351" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" s="1"/>
       <c r="B351" s="31">
         <f t="shared" si="130"/>
@@ -18186,7 +18186,7 @@
         <f t="shared" si="129"/>
         <v>13.3.0</v>
       </c>
-      <c r="G351" s="10" t="s">
+      <c r="G351" s="19" t="s">
         <v>89</v>
       </c>
       <c r="H351" s="19" t="s">
@@ -18210,7 +18210,7 @@
       <c r="N351" s="1"/>
       <c r="O351" s="1"/>
     </row>
-    <row r="352" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" s="1"/>
       <c r="B352" s="31">
         <f t="shared" si="130"/>
@@ -18255,7 +18255,7 @@
       <c r="N352" s="1"/>
       <c r="O352" s="1"/>
     </row>
-    <row r="353" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" s="1"/>
       <c r="B353" s="31">
         <f t="shared" si="130"/>
@@ -18300,7 +18300,7 @@
       <c r="N353" s="1"/>
       <c r="O353" s="1"/>
     </row>
-    <row r="354" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" s="1"/>
       <c r="B354" s="31">
         <f t="shared" si="130"/>
@@ -18345,7 +18345,7 @@
       <c r="N354" s="1"/>
       <c r="O354" s="1"/>
     </row>
-    <row r="355" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" s="1"/>
       <c r="B355" s="31">
         <f t="shared" si="130"/>
@@ -18390,7 +18390,7 @@
       <c r="N355" s="1"/>
       <c r="O355" s="1"/>
     </row>
-    <row r="356" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" s="1"/>
       <c r="B356" s="31">
         <f t="shared" si="130"/>
@@ -18435,7 +18435,7 @@
       <c r="N356" s="1"/>
       <c r="O356" s="1"/>
     </row>
-    <row r="357" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" s="1"/>
       <c r="B357" s="31">
         <f t="shared" si="130"/>
@@ -18480,7 +18480,7 @@
       <c r="N357" s="1"/>
       <c r="O357" s="1"/>
     </row>
-    <row r="358" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" s="1"/>
       <c r="B358" s="31">
         <f t="shared" si="130"/>
@@ -18525,7 +18525,7 @@
       <c r="N358" s="1"/>
       <c r="O358" s="1"/>
     </row>
-    <row r="359" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" s="1"/>
       <c r="B359" s="31">
         <f t="shared" si="130"/>
@@ -18569,7 +18569,7 @@
       <c r="N359" s="1"/>
       <c r="O359" s="1"/>
     </row>
-    <row r="360" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" s="1"/>
       <c r="B360" s="31">
         <f t="shared" ref="B360:B374" si="135">+B359+1</f>
@@ -18577,7 +18577,7 @@
       </c>
       <c r="C360" s="23">
         <f>INDEX(Lists!$D$5:$D$21,MATCH(G360,Lists!$E$5:$E$21,0))</f>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D360" s="33">
         <v>0</v>
@@ -18587,10 +18587,10 @@
       </c>
       <c r="F360" s="32" t="str">
         <f t="shared" si="134"/>
-        <v>2.0.0</v>
+        <v>15.0.0</v>
       </c>
       <c r="G360" s="10" t="s">
-        <v>570</v>
+        <v>130</v>
       </c>
       <c r="H360" s="19" t="s">
         <v>568</v>
@@ -18613,7 +18613,7 @@
       <c r="N360" s="1"/>
       <c r="O360" s="1"/>
     </row>
-    <row r="361" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" s="1"/>
       <c r="B361" s="31">
         <f t="shared" si="135"/>
@@ -18657,7 +18657,7 @@
       <c r="N361" s="1"/>
       <c r="O361" s="1"/>
     </row>
-    <row r="362" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" s="1"/>
       <c r="B362" s="31">
         <f t="shared" si="135"/>
@@ -18745,7 +18745,7 @@
       <c r="N363" s="1"/>
       <c r="O363" s="1"/>
     </row>
-    <row r="364" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364" s="1"/>
       <c r="B364" s="31">
         <f t="shared" si="135"/>
@@ -18789,7 +18789,7 @@
       <c r="N364" s="1"/>
       <c r="O364" s="1"/>
     </row>
-    <row r="365" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" s="1"/>
       <c r="B365" s="31">
         <f t="shared" si="135"/>
@@ -18833,7 +18833,7 @@
       <c r="N365" s="1"/>
       <c r="O365" s="1"/>
     </row>
-    <row r="366" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" s="1"/>
       <c r="B366" s="31">
         <f t="shared" si="135"/>
@@ -18877,7 +18877,7 @@
       <c r="N366" s="1"/>
       <c r="O366" s="1"/>
     </row>
-    <row r="367" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367" s="1"/>
       <c r="B367" s="31">
         <f t="shared" si="135"/>
@@ -18921,7 +18921,7 @@
       <c r="N367" s="1"/>
       <c r="O367" s="1"/>
     </row>
-    <row r="368" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" s="1"/>
       <c r="B368" s="31">
         <f t="shared" si="135"/>
@@ -18965,7 +18965,7 @@
       <c r="N368" s="1"/>
       <c r="O368" s="1"/>
     </row>
-    <row r="369" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" s="1"/>
       <c r="B369" s="31">
         <f t="shared" si="135"/>
@@ -19009,7 +19009,7 @@
       <c r="N369" s="1"/>
       <c r="O369" s="1"/>
     </row>
-    <row r="370" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" s="1"/>
       <c r="B370" s="31">
         <f t="shared" si="135"/>
@@ -19053,7 +19053,7 @@
       <c r="N370" s="1"/>
       <c r="O370" s="1"/>
     </row>
-    <row r="371" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" s="1"/>
       <c r="B371" s="31">
         <f t="shared" si="135"/>
@@ -19097,7 +19097,7 @@
       <c r="N371" s="1"/>
       <c r="O371" s="1"/>
     </row>
-    <row r="372" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" s="1"/>
       <c r="B372" s="31">
         <f t="shared" si="135"/>
@@ -19141,7 +19141,7 @@
       <c r="N372" s="1"/>
       <c r="O372" s="1"/>
     </row>
-    <row r="373" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" s="1"/>
       <c r="B373" s="31">
         <f t="shared" si="135"/>
@@ -19185,7 +19185,7 @@
       <c r="N373" s="1"/>
       <c r="O373" s="1"/>
     </row>
-    <row r="374" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" s="1"/>
       <c r="B374" s="31">
         <f t="shared" si="135"/>
@@ -19229,7 +19229,7 @@
       <c r="N374" s="1"/>
       <c r="O374" s="1"/>
     </row>
-    <row r="375" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" s="1"/>
       <c r="B375" s="1"/>
       <c r="C375" s="4"/>
@@ -19241,7 +19241,7 @@
       <c r="N375" s="1"/>
       <c r="O375" s="1"/>
     </row>
-    <row r="376" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" s="1"/>
       <c r="B376" s="1"/>
       <c r="C376" s="4"/>
@@ -19253,7 +19253,7 @@
       <c r="N376" s="1"/>
       <c r="O376" s="1"/>
     </row>
-    <row r="377" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" s="1"/>
       <c r="B377" s="1"/>
       <c r="C377" s="4"/>
@@ -19265,7 +19265,7 @@
       <c r="N377" s="1"/>
       <c r="O377" s="1"/>
     </row>
-    <row r="378" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" s="1"/>
       <c r="B378" s="1"/>
       <c r="C378" s="4"/>
@@ -19277,7 +19277,7 @@
       <c r="N378" s="1"/>
       <c r="O378" s="1"/>
     </row>
-    <row r="379" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" s="1"/>
       <c r="B379" s="1"/>
       <c r="C379" s="4"/>
@@ -19289,7 +19289,7 @@
       <c r="N379" s="1"/>
       <c r="O379" s="1"/>
     </row>
-    <row r="380" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" s="1"/>
       <c r="B380" s="1"/>
       <c r="C380" s="4"/>
@@ -19301,7 +19301,7 @@
       <c r="N380" s="1"/>
       <c r="O380" s="1"/>
     </row>
-    <row r="381" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" s="1"/>
       <c r="B381" s="1"/>
       <c r="C381" s="4"/>
@@ -19313,7 +19313,7 @@
       <c r="N381" s="1"/>
       <c r="O381" s="1"/>
     </row>
-    <row r="382" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" s="1"/>
       <c r="B382" s="1"/>
       <c r="C382" s="4"/>
@@ -19325,7 +19325,7 @@
       <c r="N382" s="1"/>
       <c r="O382" s="1"/>
     </row>
-    <row r="383" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" s="1"/>
       <c r="B383" s="1"/>
       <c r="C383" s="4"/>
@@ -19337,7 +19337,7 @@
       <c r="N383" s="1"/>
       <c r="O383" s="1"/>
     </row>
-    <row r="384" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" s="1"/>
       <c r="B384" s="1"/>
       <c r="C384" s="4"/>
@@ -19349,7 +19349,7 @@
       <c r="N384" s="1"/>
       <c r="O384" s="1"/>
     </row>
-    <row r="385" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" s="1"/>
       <c r="B385" s="1"/>
       <c r="C385" s="4"/>
@@ -19361,7 +19361,7 @@
       <c r="N385" s="1"/>
       <c r="O385" s="1"/>
     </row>
-    <row r="386" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" s="1"/>
       <c r="B386" s="1"/>
       <c r="C386" s="4"/>
@@ -19373,7 +19373,7 @@
       <c r="N386" s="1"/>
       <c r="O386" s="1"/>
     </row>
-    <row r="387" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" s="1"/>
       <c r="B387" s="1"/>
       <c r="C387" s="4"/>
@@ -19385,7 +19385,7 @@
       <c r="N387" s="1"/>
       <c r="O387" s="1"/>
     </row>
-    <row r="388" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" s="1"/>
       <c r="B388" s="1"/>
       <c r="C388" s="4"/>
@@ -19397,7 +19397,7 @@
       <c r="N388" s="1"/>
       <c r="O388" s="1"/>
     </row>
-    <row r="389" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" s="1"/>
       <c r="B389" s="1"/>
       <c r="C389" s="4"/>
@@ -19409,7 +19409,7 @@
       <c r="N389" s="1"/>
       <c r="O389" s="1"/>
     </row>
-    <row r="390" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" s="1"/>
       <c r="B390" s="1"/>
       <c r="C390" s="4"/>
@@ -29185,7 +29185,13 @@
       <c r="O1097" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="C5:N390" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}"/>
+  <autoFilter ref="C5:N390" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Funds"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="C3:E3"/>
   </mergeCells>

</xml_diff>

<commit_message>
Improves artifact loading for record shell dialogs
Refactors artifact initialization logic for create/edit dialogs to fetch and resolve artifacts based on record type, supporting companies and contacts via tailored queries. Enhances accuracy and consistency of prefilled artifact data when opening or submitting record shell dialogs, and adds robust fallback handling.
</commit_message>
<xml_diff>
--- a/docs/B10_DOS v260400 vrev.xlsx
+++ b/docs/B10_DOS v260400 vrev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erikc\Coding_Repository\ec-vc\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C08AB6-0D69-4F50-B3BE-92A048CA5905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF83FDF6-BA93-4670-B0E0-BC8693CDEE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0110398B-6F4E-42D1-8445-B061DE6C3E3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0110398B-6F4E-42D1-8445-B061DE6C3E3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokens" sheetId="1" r:id="rId1"/>
@@ -2228,7 +2228,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:O1097"/>
@@ -2346,7 +2346,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="31">
         <v>1</v>
@@ -2391,7 +2391,7 @@
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
     </row>
-    <row r="7" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="31">
         <f>+B6+1</f>
@@ -2437,7 +2437,7 @@
       <c r="N7" s="9"/>
       <c r="O7" s="9"/>
     </row>
-    <row r="8" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="31">
         <f t="shared" ref="B8:B71" si="3">+B7+1</f>
@@ -2483,7 +2483,7 @@
       <c r="N8" s="9"/>
       <c r="O8" s="9"/>
     </row>
-    <row r="9" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="31">
         <f t="shared" si="3"/>
@@ -2529,7 +2529,7 @@
       <c r="N9" s="9"/>
       <c r="O9" s="9"/>
     </row>
-    <row r="10" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="31">
         <f t="shared" si="3"/>
@@ -2575,7 +2575,7 @@
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
     </row>
-    <row r="11" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="31">
         <f t="shared" si="3"/>
@@ -2621,7 +2621,7 @@
       <c r="N11" s="9"/>
       <c r="O11" s="9"/>
     </row>
-    <row r="12" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="31">
         <f t="shared" si="3"/>
@@ -2667,7 +2667,7 @@
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
     </row>
-    <row r="13" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="31">
         <f t="shared" si="3"/>
@@ -2713,7 +2713,7 @@
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
     </row>
-    <row r="14" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="31">
         <f t="shared" si="3"/>
@@ -2759,7 +2759,7 @@
       <c r="N14" s="9"/>
       <c r="O14" s="9"/>
     </row>
-    <row r="15" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="31">
         <f t="shared" si="3"/>
@@ -2805,7 +2805,7 @@
       <c r="N15" s="9"/>
       <c r="O15" s="9"/>
     </row>
-    <row r="16" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="31">
         <f t="shared" si="3"/>
@@ -2851,7 +2851,7 @@
       <c r="N16" s="9"/>
       <c r="O16" s="9"/>
     </row>
-    <row r="17" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="31">
         <f t="shared" si="3"/>
@@ -2897,7 +2897,7 @@
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
     </row>
-    <row r="18" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="31">
         <f t="shared" si="3"/>
@@ -2943,7 +2943,7 @@
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
     </row>
-    <row r="19" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
       <c r="B19" s="31">
         <f t="shared" si="3"/>
@@ -2989,7 +2989,7 @@
       <c r="N19" s="9"/>
       <c r="O19" s="9"/>
     </row>
-    <row r="20" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="31">
         <f t="shared" si="3"/>
@@ -3035,7 +3035,7 @@
       <c r="N20" s="9"/>
       <c r="O20" s="9"/>
     </row>
-    <row r="21" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="31">
         <f t="shared" si="3"/>
@@ -3081,7 +3081,7 @@
       <c r="N21" s="9"/>
       <c r="O21" s="9"/>
     </row>
-    <row r="22" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="31">
         <f t="shared" si="3"/>
@@ -3127,7 +3127,7 @@
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
     </row>
-    <row r="23" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="31">
         <f t="shared" si="3"/>
@@ -3173,7 +3173,7 @@
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
     </row>
-    <row r="24" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="31">
         <f t="shared" si="3"/>
@@ -3219,7 +3219,7 @@
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
     </row>
-    <row r="25" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="31">
         <f t="shared" si="3"/>
@@ -3265,7 +3265,7 @@
       <c r="N25" s="9"/>
       <c r="O25" s="9"/>
     </row>
-    <row r="26" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
       <c r="B26" s="31">
         <f t="shared" si="3"/>
@@ -3311,7 +3311,7 @@
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
     </row>
-    <row r="27" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8"/>
       <c r="B27" s="31">
         <f t="shared" si="3"/>
@@ -3357,7 +3357,7 @@
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
     </row>
-    <row r="28" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8"/>
       <c r="B28" s="31">
         <f t="shared" si="3"/>
@@ -3403,7 +3403,7 @@
       <c r="N28" s="9"/>
       <c r="O28" s="9"/>
     </row>
-    <row r="29" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" s="31">
         <f t="shared" si="3"/>
@@ -4231,7 +4231,7 @@
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
     </row>
-    <row r="47" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
       <c r="B47" s="31">
         <f t="shared" si="3"/>
@@ -4277,7 +4277,7 @@
       <c r="N47" s="9"/>
       <c r="O47" s="1"/>
     </row>
-    <row r="48" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="31">
         <f t="shared" si="3"/>
@@ -4323,7 +4323,7 @@
       <c r="N48" s="9"/>
       <c r="O48" s="1"/>
     </row>
-    <row r="49" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="31">
         <f t="shared" si="3"/>
@@ -4369,7 +4369,7 @@
       <c r="N49" s="9"/>
       <c r="O49" s="1"/>
     </row>
-    <row r="50" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="31">
         <f t="shared" si="3"/>
@@ -4415,7 +4415,7 @@
       <c r="N50" s="9"/>
       <c r="O50" s="1"/>
     </row>
-    <row r="51" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A51" s="8"/>
       <c r="B51" s="31">
         <f t="shared" si="3"/>
@@ -4461,7 +4461,7 @@
       <c r="N51" s="9"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A52" s="8"/>
       <c r="B52" s="31">
         <f t="shared" si="3"/>
@@ -4507,7 +4507,7 @@
       <c r="N52" s="9"/>
       <c r="O52" s="1"/>
     </row>
-    <row r="53" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
       <c r="B53" s="31">
         <f t="shared" si="3"/>
@@ -4553,7 +4553,7 @@
       <c r="N53" s="9"/>
       <c r="O53" s="1"/>
     </row>
-    <row r="54" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
       <c r="B54" s="31">
         <f t="shared" si="3"/>
@@ -4599,7 +4599,7 @@
       <c r="N54" s="9"/>
       <c r="O54" s="1"/>
     </row>
-    <row r="55" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8"/>
       <c r="B55" s="31">
         <f t="shared" si="3"/>
@@ -4645,7 +4645,7 @@
       <c r="N55" s="9"/>
       <c r="O55" s="9"/>
     </row>
-    <row r="56" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8"/>
       <c r="B56" s="31">
         <f t="shared" si="3"/>
@@ -4691,7 +4691,7 @@
       <c r="N56" s="9"/>
       <c r="O56" s="9"/>
     </row>
-    <row r="57" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8"/>
       <c r="B57" s="31">
         <f t="shared" si="3"/>
@@ -4737,7 +4737,7 @@
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
     </row>
-    <row r="58" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8"/>
       <c r="B58" s="31">
         <f t="shared" si="3"/>
@@ -4783,7 +4783,7 @@
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
     </row>
-    <row r="59" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8"/>
       <c r="B59" s="31">
         <f t="shared" si="3"/>
@@ -4829,7 +4829,7 @@
       <c r="N59" s="9"/>
       <c r="O59" s="9"/>
     </row>
-    <row r="60" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8"/>
       <c r="B60" s="31">
         <f t="shared" si="3"/>
@@ -4875,7 +4875,7 @@
       <c r="N60" s="9"/>
       <c r="O60" s="9"/>
     </row>
-    <row r="61" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8"/>
       <c r="B61" s="31">
         <f t="shared" si="3"/>
@@ -4921,7 +4921,7 @@
       <c r="N61" s="9"/>
       <c r="O61" s="9"/>
     </row>
-    <row r="62" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8"/>
       <c r="B62" s="31">
         <f t="shared" si="3"/>
@@ -4967,7 +4967,7 @@
       <c r="N62" s="9"/>
       <c r="O62" s="9"/>
     </row>
-    <row r="63" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8"/>
       <c r="B63" s="31">
         <f t="shared" si="3"/>
@@ -5013,7 +5013,7 @@
       <c r="N63" s="9"/>
       <c r="O63" s="9"/>
     </row>
-    <row r="64" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A64" s="8"/>
       <c r="B64" s="31">
         <f t="shared" si="3"/>
@@ -5059,7 +5059,7 @@
       <c r="N64" s="9"/>
       <c r="O64" s="1"/>
     </row>
-    <row r="65" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
       <c r="B65" s="31">
         <f t="shared" si="3"/>
@@ -5105,7 +5105,7 @@
       <c r="N65" s="9"/>
       <c r="O65" s="1"/>
     </row>
-    <row r="66" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A66" s="8"/>
       <c r="B66" s="31">
         <f t="shared" si="3"/>
@@ -5151,7 +5151,7 @@
       <c r="N66" s="9"/>
       <c r="O66" s="1"/>
     </row>
-    <row r="67" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A67" s="8"/>
       <c r="B67" s="31">
         <f t="shared" si="3"/>
@@ -5197,7 +5197,7 @@
       <c r="N67" s="9"/>
       <c r="O67" s="1"/>
     </row>
-    <row r="68" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A68" s="8"/>
       <c r="B68" s="31">
         <f t="shared" si="3"/>
@@ -5243,7 +5243,7 @@
       <c r="N68" s="9"/>
       <c r="O68" s="1"/>
     </row>
-    <row r="69" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A69" s="8"/>
       <c r="B69" s="31">
         <f t="shared" si="3"/>
@@ -5289,7 +5289,7 @@
       <c r="N69" s="9"/>
       <c r="O69" s="1"/>
     </row>
-    <row r="70" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A70" s="8"/>
       <c r="B70" s="31">
         <f t="shared" si="3"/>
@@ -5335,7 +5335,7 @@
       <c r="N70" s="9"/>
       <c r="O70" s="1"/>
     </row>
-    <row r="71" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A71" s="8"/>
       <c r="B71" s="31">
         <f t="shared" si="3"/>
@@ -5381,7 +5381,7 @@
       <c r="N71" s="9"/>
       <c r="O71" s="1"/>
     </row>
-    <row r="72" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A72" s="8"/>
       <c r="B72" s="31">
         <f t="shared" ref="B72:B136" si="35">+B71+1</f>
@@ -5427,7 +5427,7 @@
       <c r="N72" s="9"/>
       <c r="O72" s="1"/>
     </row>
-    <row r="73" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A73" s="8"/>
       <c r="B73" s="31">
         <f t="shared" si="35"/>
@@ -5473,7 +5473,7 @@
       <c r="N73" s="9"/>
       <c r="O73" s="1"/>
     </row>
-    <row r="74" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A74" s="8"/>
       <c r="B74" s="31">
         <f t="shared" si="35"/>
@@ -5519,7 +5519,7 @@
       <c r="N74" s="9"/>
       <c r="O74" s="1"/>
     </row>
-    <row r="75" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>
       <c r="B75" s="31">
         <f t="shared" si="35"/>
@@ -5565,7 +5565,7 @@
       <c r="N75" s="9"/>
       <c r="O75" s="1"/>
     </row>
-    <row r="76" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A76" s="8"/>
       <c r="B76" s="31">
         <f t="shared" si="35"/>
@@ -5611,7 +5611,7 @@
       <c r="N76" s="9"/>
       <c r="O76" s="1"/>
     </row>
-    <row r="77" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A77" s="8"/>
       <c r="B77" s="31">
         <f t="shared" si="35"/>
@@ -5657,7 +5657,7 @@
       <c r="N77" s="9"/>
       <c r="O77" s="1"/>
     </row>
-    <row r="78" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A78" s="8"/>
       <c r="B78" s="31">
         <f t="shared" si="35"/>
@@ -5703,7 +5703,7 @@
       <c r="N78" s="9"/>
       <c r="O78" s="1"/>
     </row>
-    <row r="79" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A79" s="8"/>
       <c r="B79" s="31">
         <f t="shared" si="35"/>
@@ -5749,7 +5749,7 @@
       <c r="N79" s="9"/>
       <c r="O79" s="1"/>
     </row>
-    <row r="80" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A80" s="8"/>
       <c r="B80" s="31">
         <f t="shared" si="35"/>
@@ -5795,7 +5795,7 @@
       <c r="N80" s="9"/>
       <c r="O80" s="1"/>
     </row>
-    <row r="81" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A81" s="8"/>
       <c r="B81" s="31">
         <f t="shared" si="35"/>
@@ -5841,7 +5841,7 @@
       <c r="N81" s="9"/>
       <c r="O81" s="1"/>
     </row>
-    <row r="82" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A82" s="8"/>
       <c r="B82" s="31">
         <f t="shared" si="35"/>
@@ -5887,7 +5887,7 @@
       <c r="N82" s="9"/>
       <c r="O82" s="1"/>
     </row>
-    <row r="83" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A83" s="8"/>
       <c r="B83" s="31">
         <f t="shared" si="35"/>
@@ -5933,7 +5933,7 @@
       <c r="N83" s="9"/>
       <c r="O83" s="1"/>
     </row>
-    <row r="84" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A84" s="8"/>
       <c r="B84" s="31">
         <f t="shared" si="35"/>
@@ -5979,7 +5979,7 @@
       <c r="N84" s="9"/>
       <c r="O84" s="1"/>
     </row>
-    <row r="85" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A85" s="8"/>
       <c r="B85" s="31">
         <f t="shared" si="35"/>
@@ -6025,7 +6025,7 @@
       <c r="N85" s="9"/>
       <c r="O85" s="1"/>
     </row>
-    <row r="86" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A86" s="8"/>
       <c r="B86" s="31">
         <f t="shared" si="35"/>
@@ -6071,7 +6071,7 @@
       <c r="N86" s="9"/>
       <c r="O86" s="1"/>
     </row>
-    <row r="87" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A87" s="8"/>
       <c r="B87" s="31">
         <f t="shared" si="35"/>
@@ -6117,7 +6117,7 @@
       <c r="N87" s="9"/>
       <c r="O87" s="1"/>
     </row>
-    <row r="88" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A88" s="8"/>
       <c r="B88" s="31">
         <f t="shared" si="35"/>
@@ -6163,7 +6163,7 @@
       <c r="N88" s="9"/>
       <c r="O88" s="1"/>
     </row>
-    <row r="89" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A89" s="8"/>
       <c r="B89" s="31">
         <f t="shared" si="35"/>
@@ -6209,7 +6209,7 @@
       <c r="N89" s="9"/>
       <c r="O89" s="1"/>
     </row>
-    <row r="90" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A90" s="8"/>
       <c r="B90" s="31">
         <f t="shared" si="35"/>
@@ -6255,7 +6255,7 @@
       <c r="N90" s="9"/>
       <c r="O90" s="1"/>
     </row>
-    <row r="91" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A91" s="8"/>
       <c r="B91" s="31">
         <f t="shared" si="35"/>
@@ -6301,7 +6301,7 @@
       <c r="N91" s="9"/>
       <c r="O91" s="1"/>
     </row>
-    <row r="92" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A92" s="8"/>
       <c r="B92" s="31">
         <f t="shared" si="35"/>
@@ -6347,7 +6347,7 @@
       <c r="N92" s="9"/>
       <c r="O92" s="1"/>
     </row>
-    <row r="93" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A93" s="8"/>
       <c r="B93" s="31">
         <f t="shared" si="35"/>
@@ -6393,7 +6393,7 @@
       <c r="N93" s="9"/>
       <c r="O93" s="1"/>
     </row>
-    <row r="94" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A94" s="8"/>
       <c r="B94" s="31">
         <f t="shared" si="35"/>
@@ -6439,7 +6439,7 @@
       <c r="N94" s="9"/>
       <c r="O94" s="1"/>
     </row>
-    <row r="95" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A95" s="8"/>
       <c r="B95" s="31">
         <f t="shared" si="35"/>
@@ -6485,7 +6485,7 @@
       <c r="N95" s="9"/>
       <c r="O95" s="1"/>
     </row>
-    <row r="96" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A96" s="8"/>
       <c r="B96" s="31">
         <f t="shared" si="35"/>
@@ -6531,7 +6531,7 @@
       <c r="N96" s="9"/>
       <c r="O96" s="1"/>
     </row>
-    <row r="97" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A97" s="8"/>
       <c r="B97" s="31">
         <f t="shared" si="35"/>
@@ -6577,7 +6577,7 @@
       <c r="N97" s="9"/>
       <c r="O97" s="1"/>
     </row>
-    <row r="98" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A98" s="8"/>
       <c r="B98" s="31">
         <f t="shared" si="35"/>
@@ -6623,7 +6623,7 @@
       <c r="N98" s="9"/>
       <c r="O98" s="1"/>
     </row>
-    <row r="99" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A99" s="8"/>
       <c r="B99" s="31">
         <f t="shared" si="35"/>
@@ -6669,7 +6669,7 @@
       <c r="N99" s="9"/>
       <c r="O99" s="1"/>
     </row>
-    <row r="100" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A100" s="8"/>
       <c r="B100" s="31">
         <f t="shared" si="35"/>
@@ -6715,7 +6715,7 @@
       <c r="N100" s="9"/>
       <c r="O100" s="1"/>
     </row>
-    <row r="101" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A101" s="8"/>
       <c r="B101" s="31">
         <f t="shared" ref="B101:B102" si="41">+B100+1</f>
@@ -6761,7 +6761,7 @@
       <c r="N101" s="9"/>
       <c r="O101" s="1"/>
     </row>
-    <row r="102" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A102" s="8"/>
       <c r="B102" s="31">
         <f t="shared" si="41"/>
@@ -6807,7 +6807,7 @@
       <c r="N102" s="9"/>
       <c r="O102" s="1"/>
     </row>
-    <row r="103" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A103" s="8"/>
       <c r="B103" s="31">
         <f t="shared" si="35"/>
@@ -6853,7 +6853,7 @@
       <c r="N103" s="9"/>
       <c r="O103" s="1"/>
     </row>
-    <row r="104" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A104" s="8"/>
       <c r="B104" s="31">
         <f t="shared" si="35"/>
@@ -6899,7 +6899,7 @@
       <c r="N104" s="9"/>
       <c r="O104" s="1"/>
     </row>
-    <row r="105" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A105" s="8"/>
       <c r="B105" s="31">
         <f t="shared" si="35"/>
@@ -6945,7 +6945,7 @@
       <c r="N105" s="9"/>
       <c r="O105" s="1"/>
     </row>
-    <row r="106" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A106" s="8"/>
       <c r="B106" s="31">
         <f t="shared" si="35"/>
@@ -6991,7 +6991,7 @@
       <c r="N106" s="9"/>
       <c r="O106" s="1"/>
     </row>
-    <row r="107" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A107" s="8"/>
       <c r="B107" s="31">
         <f t="shared" si="35"/>
@@ -7037,7 +7037,7 @@
       <c r="N107" s="9"/>
       <c r="O107" s="1"/>
     </row>
-    <row r="108" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A108" s="8"/>
       <c r="B108" s="31">
         <f t="shared" si="35"/>
@@ -7083,7 +7083,7 @@
       <c r="N108" s="9"/>
       <c r="O108" s="1"/>
     </row>
-    <row r="109" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A109" s="8"/>
       <c r="B109" s="31">
         <f t="shared" si="35"/>
@@ -7129,7 +7129,7 @@
       <c r="N109" s="9"/>
       <c r="O109" s="1"/>
     </row>
-    <row r="110" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A110" s="8"/>
       <c r="B110" s="31">
         <f t="shared" si="35"/>
@@ -7175,7 +7175,7 @@
       <c r="N110" s="9"/>
       <c r="O110" s="1"/>
     </row>
-    <row r="111" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A111" s="8"/>
       <c r="B111" s="31">
         <f t="shared" si="35"/>
@@ -7221,7 +7221,7 @@
       <c r="N111" s="9"/>
       <c r="O111" s="1"/>
     </row>
-    <row r="112" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A112" s="8"/>
       <c r="B112" s="31">
         <f t="shared" si="35"/>
@@ -7267,7 +7267,7 @@
       <c r="N112" s="9"/>
       <c r="O112" s="1"/>
     </row>
-    <row r="113" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A113" s="8"/>
       <c r="B113" s="31">
         <f t="shared" si="35"/>
@@ -7313,7 +7313,7 @@
       <c r="N113" s="9"/>
       <c r="O113" s="1"/>
     </row>
-    <row r="114" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A114" s="8"/>
       <c r="B114" s="31">
         <f t="shared" si="35"/>
@@ -7359,7 +7359,7 @@
       <c r="N114" s="9"/>
       <c r="O114" s="1"/>
     </row>
-    <row r="115" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A115" s="8"/>
       <c r="B115" s="31">
         <f t="shared" si="35"/>
@@ -7405,7 +7405,7 @@
       <c r="N115" s="9"/>
       <c r="O115" s="1"/>
     </row>
-    <row r="116" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A116" s="8"/>
       <c r="B116" s="31">
         <f t="shared" si="35"/>
@@ -7451,7 +7451,7 @@
       <c r="N116" s="9"/>
       <c r="O116" s="1"/>
     </row>
-    <row r="117" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A117" s="8"/>
       <c r="B117" s="31">
         <f t="shared" si="35"/>
@@ -7497,7 +7497,7 @@
       <c r="N117" s="9"/>
       <c r="O117" s="1"/>
     </row>
-    <row r="118" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A118" s="8"/>
       <c r="B118" s="31">
         <f t="shared" si="35"/>
@@ -7543,7 +7543,7 @@
       <c r="N118" s="9"/>
       <c r="O118" s="1"/>
     </row>
-    <row r="119" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A119" s="8"/>
       <c r="B119" s="31">
         <f t="shared" si="35"/>
@@ -7589,7 +7589,7 @@
       <c r="N119" s="9"/>
       <c r="O119" s="1"/>
     </row>
-    <row r="120" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A120" s="8"/>
       <c r="B120" s="31">
         <f t="shared" si="35"/>
@@ -7635,7 +7635,7 @@
       <c r="N120" s="9"/>
       <c r="O120" s="1"/>
     </row>
-    <row r="121" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A121" s="8"/>
       <c r="B121" s="31">
         <f t="shared" si="35"/>
@@ -7681,7 +7681,7 @@
       <c r="N121" s="9"/>
       <c r="O121" s="1"/>
     </row>
-    <row r="122" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8"/>
       <c r="B122" s="31">
         <f t="shared" si="35"/>
@@ -7727,7 +7727,7 @@
       <c r="N122" s="9"/>
       <c r="O122" s="1"/>
     </row>
-    <row r="123" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A123" s="8"/>
       <c r="B123" s="31">
         <f t="shared" si="35"/>
@@ -7773,7 +7773,7 @@
       <c r="N123" s="9"/>
       <c r="O123" s="1"/>
     </row>
-    <row r="124" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A124" s="8"/>
       <c r="B124" s="31">
         <f t="shared" si="35"/>
@@ -7819,7 +7819,7 @@
       <c r="N124" s="9"/>
       <c r="O124" s="1"/>
     </row>
-    <row r="125" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A125" s="8"/>
       <c r="B125" s="31">
         <f t="shared" si="35"/>
@@ -7865,7 +7865,7 @@
       <c r="N125" s="9"/>
       <c r="O125" s="1"/>
     </row>
-    <row r="126" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A126" s="8"/>
       <c r="B126" s="31">
         <f t="shared" si="35"/>
@@ -7911,7 +7911,7 @@
       <c r="N126" s="9"/>
       <c r="O126" s="1"/>
     </row>
-    <row r="127" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A127" s="8"/>
       <c r="B127" s="31">
         <f t="shared" si="35"/>
@@ -7957,7 +7957,7 @@
       <c r="N127" s="9"/>
       <c r="O127" s="1"/>
     </row>
-    <row r="128" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A128" s="8"/>
       <c r="B128" s="31">
         <f t="shared" si="35"/>
@@ -8003,7 +8003,7 @@
       <c r="N128" s="9"/>
       <c r="O128" s="1"/>
     </row>
-    <row r="129" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A129" s="8"/>
       <c r="B129" s="31">
         <f t="shared" si="35"/>
@@ -8049,7 +8049,7 @@
       <c r="N129" s="9"/>
       <c r="O129" s="1"/>
     </row>
-    <row r="130" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A130" s="8"/>
       <c r="B130" s="31">
         <f t="shared" si="35"/>
@@ -8095,7 +8095,7 @@
       <c r="N130" s="9"/>
       <c r="O130" s="1"/>
     </row>
-    <row r="131" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A131" s="8"/>
       <c r="B131" s="31">
         <f t="shared" si="35"/>
@@ -8141,7 +8141,7 @@
       <c r="N131" s="9"/>
       <c r="O131" s="1"/>
     </row>
-    <row r="132" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A132" s="8"/>
       <c r="B132" s="31">
         <f t="shared" si="35"/>
@@ -8187,7 +8187,7 @@
       <c r="N132" s="9"/>
       <c r="O132" s="1"/>
     </row>
-    <row r="133" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A133" s="8"/>
       <c r="B133" s="31">
         <f t="shared" si="35"/>
@@ -8233,7 +8233,7 @@
       <c r="N133" s="9"/>
       <c r="O133" s="1"/>
     </row>
-    <row r="134" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
       <c r="B134" s="31">
         <f t="shared" si="35"/>
@@ -8279,7 +8279,7 @@
       <c r="N134" s="9"/>
       <c r="O134" s="1"/>
     </row>
-    <row r="135" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1"/>
       <c r="B135" s="31">
         <f t="shared" si="35"/>
@@ -8325,7 +8325,7 @@
       <c r="N135" s="9"/>
       <c r="O135" s="1"/>
     </row>
-    <row r="136" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1"/>
       <c r="B136" s="31">
         <f t="shared" si="35"/>
@@ -8371,7 +8371,7 @@
       <c r="N136" s="9"/>
       <c r="O136" s="1"/>
     </row>
-    <row r="137" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1"/>
       <c r="B137" s="31">
         <f t="shared" ref="B137:B200" si="52">+B136+1</f>
@@ -8417,7 +8417,7 @@
       <c r="N137" s="9"/>
       <c r="O137" s="1"/>
     </row>
-    <row r="138" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1"/>
       <c r="B138" s="31">
         <f t="shared" si="52"/>
@@ -8463,7 +8463,7 @@
       <c r="N138" s="9"/>
       <c r="O138" s="1"/>
     </row>
-    <row r="139" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1"/>
       <c r="B139" s="31">
         <f t="shared" si="52"/>
@@ -8509,7 +8509,7 @@
       <c r="N139" s="9"/>
       <c r="O139" s="1"/>
     </row>
-    <row r="140" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A140" s="8"/>
       <c r="B140" s="31">
         <f t="shared" si="52"/>
@@ -8555,7 +8555,7 @@
       <c r="N140" s="9"/>
       <c r="O140" s="9"/>
     </row>
-    <row r="141" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A141" s="8"/>
       <c r="B141" s="31">
         <f t="shared" si="52"/>
@@ -8601,7 +8601,7 @@
       <c r="N141" s="9"/>
       <c r="O141" s="9"/>
     </row>
-    <row r="142" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A142" s="8"/>
       <c r="B142" s="31">
         <f t="shared" si="52"/>
@@ -8647,7 +8647,7 @@
       <c r="N142" s="9"/>
       <c r="O142" s="9"/>
     </row>
-    <row r="143" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A143" s="8"/>
       <c r="B143" s="31">
         <f t="shared" si="52"/>
@@ -8693,7 +8693,7 @@
       <c r="N143" s="9"/>
       <c r="O143" s="9"/>
     </row>
-    <row r="144" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A144" s="8"/>
       <c r="B144" s="31">
         <f t="shared" si="52"/>
@@ -8739,7 +8739,7 @@
       <c r="N144" s="9"/>
       <c r="O144" s="9"/>
     </row>
-    <row r="145" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A145" s="8"/>
       <c r="B145" s="31">
         <f t="shared" si="52"/>
@@ -8785,7 +8785,7 @@
       <c r="N145" s="9"/>
       <c r="O145" s="9"/>
     </row>
-    <row r="146" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A146" s="8"/>
       <c r="B146" s="31">
         <f t="shared" si="52"/>
@@ -8831,7 +8831,7 @@
       <c r="N146" s="9"/>
       <c r="O146" s="9"/>
     </row>
-    <row r="147" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A147" s="8"/>
       <c r="B147" s="31">
         <f t="shared" si="52"/>
@@ -8877,7 +8877,7 @@
       <c r="N147" s="9"/>
       <c r="O147" s="9"/>
     </row>
-    <row r="148" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A148" s="8"/>
       <c r="B148" s="31">
         <f t="shared" si="52"/>
@@ -8923,7 +8923,7 @@
       <c r="N148" s="9"/>
       <c r="O148" s="9"/>
     </row>
-    <row r="149" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1"/>
       <c r="B149" s="31">
         <f t="shared" si="52"/>
@@ -8969,7 +8969,7 @@
       <c r="N149" s="9"/>
       <c r="O149" s="1"/>
     </row>
-    <row r="150" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1"/>
       <c r="B150" s="31">
         <f t="shared" si="52"/>
@@ -9015,7 +9015,7 @@
       <c r="N150" s="9"/>
       <c r="O150" s="1"/>
     </row>
-    <row r="151" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1"/>
       <c r="B151" s="31">
         <f t="shared" si="52"/>
@@ -9061,7 +9061,7 @@
       <c r="N151" s="9"/>
       <c r="O151" s="1"/>
     </row>
-    <row r="152" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1"/>
       <c r="B152" s="31">
         <f t="shared" si="52"/>
@@ -9107,7 +9107,7 @@
       <c r="N152" s="9"/>
       <c r="O152" s="1"/>
     </row>
-    <row r="153" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1"/>
       <c r="B153" s="31">
         <f t="shared" si="52"/>
@@ -9153,7 +9153,7 @@
       <c r="N153" s="9"/>
       <c r="O153" s="1"/>
     </row>
-    <row r="154" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1"/>
       <c r="B154" s="31">
         <f t="shared" si="52"/>
@@ -9199,7 +9199,7 @@
       <c r="N154" s="9"/>
       <c r="O154" s="1"/>
     </row>
-    <row r="155" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1"/>
       <c r="B155" s="31">
         <f t="shared" si="52"/>
@@ -9245,7 +9245,7 @@
       <c r="N155" s="9"/>
       <c r="O155" s="1"/>
     </row>
-    <row r="156" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1"/>
       <c r="B156" s="31">
         <f t="shared" si="52"/>
@@ -9291,7 +9291,7 @@
       <c r="N156" s="9"/>
       <c r="O156" s="1"/>
     </row>
-    <row r="157" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1"/>
       <c r="B157" s="31">
         <f t="shared" si="52"/>
@@ -9337,7 +9337,7 @@
       <c r="N157" s="9"/>
       <c r="O157" s="1"/>
     </row>
-    <row r="158" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A158" s="1"/>
       <c r="B158" s="31">
         <f t="shared" si="52"/>
@@ -9383,7 +9383,7 @@
       <c r="N158" s="9"/>
       <c r="O158" s="1"/>
     </row>
-    <row r="159" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A159" s="1"/>
       <c r="B159" s="31">
         <f t="shared" si="52"/>
@@ -9429,7 +9429,7 @@
       <c r="N159" s="9"/>
       <c r="O159" s="1"/>
     </row>
-    <row r="160" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A160" s="1"/>
       <c r="B160" s="31">
         <f t="shared" si="52"/>
@@ -9475,7 +9475,7 @@
       <c r="N160" s="9"/>
       <c r="O160" s="1"/>
     </row>
-    <row r="161" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1"/>
       <c r="B161" s="31">
         <f t="shared" si="52"/>
@@ -9521,7 +9521,7 @@
       <c r="N161" s="9"/>
       <c r="O161" s="1"/>
     </row>
-    <row r="162" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A162" s="1"/>
       <c r="B162" s="31">
         <f t="shared" si="52"/>
@@ -9567,7 +9567,7 @@
       <c r="N162" s="9"/>
       <c r="O162" s="1"/>
     </row>
-    <row r="163" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A163" s="1"/>
       <c r="B163" s="31">
         <f t="shared" si="52"/>
@@ -9613,7 +9613,7 @@
       <c r="N163" s="9"/>
       <c r="O163" s="1"/>
     </row>
-    <row r="164" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A164" s="1"/>
       <c r="B164" s="31">
         <f t="shared" si="52"/>
@@ -9659,7 +9659,7 @@
       <c r="N164" s="9"/>
       <c r="O164" s="1"/>
     </row>
-    <row r="165" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1"/>
       <c r="B165" s="31">
         <f t="shared" si="52"/>
@@ -9705,7 +9705,7 @@
       <c r="N165" s="9"/>
       <c r="O165" s="1"/>
     </row>
-    <row r="166" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A166" s="1"/>
       <c r="B166" s="31">
         <f t="shared" si="52"/>
@@ -9751,7 +9751,7 @@
       <c r="N166" s="9"/>
       <c r="O166" s="1"/>
     </row>
-    <row r="167" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A167" s="1"/>
       <c r="B167" s="31">
         <f t="shared" si="52"/>
@@ -9797,7 +9797,7 @@
       <c r="N167" s="9"/>
       <c r="O167" s="1"/>
     </row>
-    <row r="168" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A168" s="1"/>
       <c r="B168" s="31">
         <f t="shared" si="52"/>
@@ -9843,7 +9843,7 @@
       <c r="N168" s="9"/>
       <c r="O168" s="1"/>
     </row>
-    <row r="169" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A169" s="1"/>
       <c r="B169" s="31">
         <f t="shared" si="52"/>
@@ -9889,7 +9889,7 @@
       <c r="N169" s="9"/>
       <c r="O169" s="1"/>
     </row>
-    <row r="170" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A170" s="1"/>
       <c r="B170" s="31">
         <f t="shared" si="52"/>
@@ -9935,7 +9935,7 @@
       <c r="N170" s="9"/>
       <c r="O170" s="1"/>
     </row>
-    <row r="171" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A171" s="1"/>
       <c r="B171" s="31">
         <f t="shared" si="52"/>
@@ -9981,7 +9981,7 @@
       <c r="N171" s="9"/>
       <c r="O171" s="1"/>
     </row>
-    <row r="172" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A172" s="1"/>
       <c r="B172" s="31">
         <f t="shared" si="52"/>
@@ -10027,7 +10027,7 @@
       <c r="N172" s="9"/>
       <c r="O172" s="1"/>
     </row>
-    <row r="173" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A173" s="1"/>
       <c r="B173" s="31">
         <f t="shared" si="52"/>
@@ -10073,7 +10073,7 @@
       <c r="N173" s="9"/>
       <c r="O173" s="1"/>
     </row>
-    <row r="174" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A174" s="8"/>
       <c r="B174" s="31">
         <f t="shared" si="52"/>
@@ -10119,7 +10119,7 @@
       <c r="N174" s="9"/>
       <c r="O174" s="1"/>
     </row>
-    <row r="175" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A175" s="8"/>
       <c r="B175" s="31">
         <f t="shared" si="52"/>
@@ -10165,7 +10165,7 @@
       <c r="N175" s="9"/>
       <c r="O175" s="1"/>
     </row>
-    <row r="176" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A176" s="8"/>
       <c r="B176" s="31">
         <f t="shared" si="52"/>
@@ -10211,7 +10211,7 @@
       <c r="N176" s="9"/>
       <c r="O176" s="1"/>
     </row>
-    <row r="177" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A177" s="8"/>
       <c r="B177" s="31">
         <f t="shared" si="52"/>
@@ -10257,7 +10257,7 @@
       <c r="N177" s="9"/>
       <c r="O177" s="1"/>
     </row>
-    <row r="178" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A178" s="8"/>
       <c r="B178" s="31">
         <f t="shared" si="52"/>
@@ -10303,7 +10303,7 @@
       <c r="N178" s="9"/>
       <c r="O178" s="1"/>
     </row>
-    <row r="179" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A179" s="8"/>
       <c r="B179" s="31">
         <f t="shared" si="52"/>
@@ -10349,7 +10349,7 @@
       <c r="N179" s="9"/>
       <c r="O179" s="9"/>
     </row>
-    <row r="180" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A180" s="8"/>
       <c r="B180" s="31">
         <f t="shared" si="52"/>
@@ -10395,7 +10395,7 @@
       <c r="N180" s="9"/>
       <c r="O180" s="9"/>
     </row>
-    <row r="181" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A181" s="8"/>
       <c r="B181" s="31">
         <f t="shared" si="52"/>
@@ -10441,7 +10441,7 @@
       <c r="N181" s="9"/>
       <c r="O181" s="9"/>
     </row>
-    <row r="182" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A182" s="8"/>
       <c r="B182" s="31">
         <f t="shared" si="52"/>
@@ -10487,7 +10487,7 @@
       <c r="N182" s="9"/>
       <c r="O182" s="9"/>
     </row>
-    <row r="183" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8"/>
       <c r="B183" s="31">
         <f t="shared" si="52"/>
@@ -10533,7 +10533,7 @@
       <c r="N183" s="9"/>
       <c r="O183" s="9"/>
     </row>
-    <row r="184" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A184" s="8"/>
       <c r="B184" s="31">
         <f t="shared" si="52"/>
@@ -10579,7 +10579,7 @@
       <c r="N184" s="9"/>
       <c r="O184" s="9"/>
     </row>
-    <row r="185" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8"/>
       <c r="B185" s="31">
         <f t="shared" si="52"/>
@@ -10625,7 +10625,7 @@
       <c r="N185" s="9"/>
       <c r="O185" s="9"/>
     </row>
-    <row r="186" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A186" s="8"/>
       <c r="B186" s="31">
         <f t="shared" si="52"/>
@@ -10671,7 +10671,7 @@
       <c r="N186" s="9"/>
       <c r="O186" s="9"/>
     </row>
-    <row r="187" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A187" s="8"/>
       <c r="B187" s="31">
         <f t="shared" si="52"/>
@@ -10717,7 +10717,7 @@
       <c r="N187" s="9"/>
       <c r="O187" s="1"/>
     </row>
-    <row r="188" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A188" s="8"/>
       <c r="B188" s="31">
         <f t="shared" si="52"/>
@@ -10763,7 +10763,7 @@
       <c r="N188" s="9"/>
       <c r="O188" s="1"/>
     </row>
-    <row r="189" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A189" s="8"/>
       <c r="B189" s="31">
         <f t="shared" si="52"/>
@@ -10809,7 +10809,7 @@
       <c r="N189" s="9"/>
       <c r="O189" s="1"/>
     </row>
-    <row r="190" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A190" s="8"/>
       <c r="B190" s="31">
         <f t="shared" si="52"/>
@@ -10855,7 +10855,7 @@
       <c r="N190" s="9"/>
       <c r="O190" s="1"/>
     </row>
-    <row r="191" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A191" s="8"/>
       <c r="B191" s="31">
         <f t="shared" si="52"/>
@@ -10901,7 +10901,7 @@
       <c r="N191" s="9"/>
       <c r="O191" s="1"/>
     </row>
-    <row r="192" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A192" s="8"/>
       <c r="B192" s="31">
         <f t="shared" si="52"/>
@@ -10947,7 +10947,7 @@
       <c r="N192" s="9"/>
       <c r="O192" s="1"/>
     </row>
-    <row r="193" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A193" s="8"/>
       <c r="B193" s="31">
         <f t="shared" si="52"/>
@@ -10993,7 +10993,7 @@
       <c r="N193" s="9"/>
       <c r="O193" s="1"/>
     </row>
-    <row r="194" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A194" s="8"/>
       <c r="B194" s="31">
         <f t="shared" si="52"/>
@@ -11039,7 +11039,7 @@
       <c r="N194" s="9"/>
       <c r="O194" s="1"/>
     </row>
-    <row r="195" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A195" s="8"/>
       <c r="B195" s="31">
         <f t="shared" si="52"/>
@@ -11085,7 +11085,7 @@
       <c r="N195" s="9"/>
       <c r="O195" s="1"/>
     </row>
-    <row r="196" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A196" s="8"/>
       <c r="B196" s="31">
         <f t="shared" si="52"/>
@@ -11131,7 +11131,7 @@
       <c r="N196" s="9"/>
       <c r="O196" s="1"/>
     </row>
-    <row r="197" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A197" s="8"/>
       <c r="B197" s="31">
         <f t="shared" si="52"/>
@@ -11177,7 +11177,7 @@
       <c r="N197" s="9"/>
       <c r="O197" s="1"/>
     </row>
-    <row r="198" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A198" s="8"/>
       <c r="B198" s="31">
         <f t="shared" si="52"/>
@@ -11223,7 +11223,7 @@
       <c r="N198" s="9"/>
       <c r="O198" s="1"/>
     </row>
-    <row r="199" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A199" s="8"/>
       <c r="B199" s="31">
         <f t="shared" si="52"/>
@@ -11269,7 +11269,7 @@
       <c r="N199" s="9"/>
       <c r="O199" s="1"/>
     </row>
-    <row r="200" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A200" s="8"/>
       <c r="B200" s="31">
         <f t="shared" si="52"/>
@@ -11315,7 +11315,7 @@
       <c r="N200" s="9"/>
       <c r="O200" s="1"/>
     </row>
-    <row r="201" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A201" s="8"/>
       <c r="B201" s="31">
         <f t="shared" ref="B201:B264" si="87">+B200+1</f>
@@ -11361,7 +11361,7 @@
       <c r="N201" s="9"/>
       <c r="O201" s="1"/>
     </row>
-    <row r="202" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A202" s="8"/>
       <c r="B202" s="31">
         <f t="shared" si="87"/>
@@ -11407,7 +11407,7 @@
       <c r="N202" s="9"/>
       <c r="O202" s="1"/>
     </row>
-    <row r="203" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A203" s="1"/>
       <c r="B203" s="31">
         <f t="shared" si="87"/>
@@ -11453,7 +11453,7 @@
       <c r="N203" s="9"/>
       <c r="O203" s="1"/>
     </row>
-    <row r="204" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A204" s="1"/>
       <c r="B204" s="31">
         <f t="shared" si="87"/>
@@ -11499,7 +11499,7 @@
       <c r="N204" s="9"/>
       <c r="O204" s="1"/>
     </row>
-    <row r="205" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A205" s="1"/>
       <c r="B205" s="31">
         <f t="shared" si="87"/>
@@ -11545,7 +11545,7 @@
       <c r="N205" s="9"/>
       <c r="O205" s="1"/>
     </row>
-    <row r="206" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A206" s="1"/>
       <c r="B206" s="31">
         <f t="shared" si="87"/>
@@ -11591,7 +11591,7 @@
       <c r="N206" s="9"/>
       <c r="O206" s="1"/>
     </row>
-    <row r="207" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A207" s="1"/>
       <c r="B207" s="31">
         <f t="shared" si="87"/>
@@ -11637,7 +11637,7 @@
       <c r="N207" s="9"/>
       <c r="O207" s="1"/>
     </row>
-    <row r="208" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A208" s="1"/>
       <c r="B208" s="31">
         <f t="shared" si="87"/>
@@ -11683,7 +11683,7 @@
       <c r="N208" s="9"/>
       <c r="O208" s="1"/>
     </row>
-    <row r="209" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A209" s="1"/>
       <c r="B209" s="31">
         <f t="shared" si="87"/>
@@ -11729,7 +11729,7 @@
       <c r="N209" s="9"/>
       <c r="O209" s="1"/>
     </row>
-    <row r="210" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A210" s="1"/>
       <c r="B210" s="31">
         <f t="shared" si="87"/>
@@ -11775,7 +11775,7 @@
       <c r="N210" s="9"/>
       <c r="O210" s="1"/>
     </row>
-    <row r="211" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A211" s="1"/>
       <c r="B211" s="31">
         <f t="shared" si="87"/>
@@ -11821,7 +11821,7 @@
       <c r="N211" s="9"/>
       <c r="O211" s="1"/>
     </row>
-    <row r="212" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A212" s="8"/>
       <c r="B212" s="31">
         <f t="shared" si="87"/>
@@ -11867,7 +11867,7 @@
       <c r="N212" s="9"/>
       <c r="O212" s="9"/>
     </row>
-    <row r="213" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A213" s="8"/>
       <c r="B213" s="31">
         <f t="shared" si="87"/>
@@ -11913,7 +11913,7 @@
       <c r="N213" s="9"/>
       <c r="O213" s="9"/>
     </row>
-    <row r="214" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A214" s="8"/>
       <c r="B214" s="31">
         <f t="shared" si="87"/>
@@ -11959,7 +11959,7 @@
       <c r="N214" s="9"/>
       <c r="O214" s="9"/>
     </row>
-    <row r="215" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A215" s="8"/>
       <c r="B215" s="31">
         <f t="shared" si="87"/>
@@ -12005,7 +12005,7 @@
       <c r="N215" s="9"/>
       <c r="O215" s="9"/>
     </row>
-    <row r="216" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A216" s="8"/>
       <c r="B216" s="31">
         <f t="shared" si="87"/>
@@ -12051,7 +12051,7 @@
       <c r="N216" s="9"/>
       <c r="O216" s="9"/>
     </row>
-    <row r="217" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A217" s="8"/>
       <c r="B217" s="31">
         <f t="shared" si="87"/>
@@ -12097,7 +12097,7 @@
       <c r="N217" s="9"/>
       <c r="O217" s="9"/>
     </row>
-    <row r="218" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A218" s="8"/>
       <c r="B218" s="31">
         <f t="shared" si="87"/>
@@ -12143,7 +12143,7 @@
       <c r="N218" s="9"/>
       <c r="O218" s="9"/>
     </row>
-    <row r="219" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A219" s="8"/>
       <c r="B219" s="31">
         <f t="shared" si="87"/>
@@ -12189,7 +12189,7 @@
       <c r="N219" s="9"/>
       <c r="O219" s="9"/>
     </row>
-    <row r="220" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A220" s="8"/>
       <c r="B220" s="31">
         <f t="shared" si="87"/>
@@ -12235,7 +12235,7 @@
       <c r="N220" s="9"/>
       <c r="O220" s="9"/>
     </row>
-    <row r="221" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A221" s="1"/>
       <c r="B221" s="31">
         <f t="shared" si="87"/>
@@ -12281,7 +12281,7 @@
       <c r="N221" s="9"/>
       <c r="O221" s="1"/>
     </row>
-    <row r="222" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A222" s="1"/>
       <c r="B222" s="31">
         <f t="shared" si="87"/>
@@ -12327,7 +12327,7 @@
       <c r="N222" s="9"/>
       <c r="O222" s="1"/>
     </row>
-    <row r="223" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A223" s="1"/>
       <c r="B223" s="31">
         <f t="shared" si="87"/>
@@ -12373,7 +12373,7 @@
       <c r="N223" s="9"/>
       <c r="O223" s="1"/>
     </row>
-    <row r="224" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A224" s="1"/>
       <c r="B224" s="31">
         <f t="shared" si="87"/>
@@ -12419,7 +12419,7 @@
       <c r="N224" s="9"/>
       <c r="O224" s="1"/>
     </row>
-    <row r="225" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A225" s="1"/>
       <c r="B225" s="31">
         <f t="shared" si="87"/>
@@ -12465,7 +12465,7 @@
       <c r="N225" s="9"/>
       <c r="O225" s="1"/>
     </row>
-    <row r="226" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A226" s="1"/>
       <c r="B226" s="31">
         <f t="shared" si="87"/>
@@ -12511,7 +12511,7 @@
       <c r="N226" s="9"/>
       <c r="O226" s="1"/>
     </row>
-    <row r="227" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A227" s="1"/>
       <c r="B227" s="31">
         <f t="shared" si="87"/>
@@ -12557,7 +12557,7 @@
       <c r="N227" s="9"/>
       <c r="O227" s="1"/>
     </row>
-    <row r="228" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A228" s="1"/>
       <c r="B228" s="31">
         <f t="shared" si="87"/>
@@ -12603,7 +12603,7 @@
       <c r="N228" s="9"/>
       <c r="O228" s="1"/>
     </row>
-    <row r="229" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A229" s="1"/>
       <c r="B229" s="31">
         <f t="shared" si="87"/>
@@ -12649,7 +12649,7 @@
       <c r="N229" s="9"/>
       <c r="O229" s="1"/>
     </row>
-    <row r="230" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A230" s="1"/>
       <c r="B230" s="31">
         <f t="shared" si="87"/>
@@ -12695,7 +12695,7 @@
       <c r="N230" s="9"/>
       <c r="O230" s="1"/>
     </row>
-    <row r="231" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A231" s="1"/>
       <c r="B231" s="31">
         <f t="shared" si="87"/>
@@ -12741,7 +12741,7 @@
       <c r="N231" s="9"/>
       <c r="O231" s="1"/>
     </row>
-    <row r="232" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A232" s="1"/>
       <c r="B232" s="31">
         <f t="shared" si="87"/>
@@ -12787,7 +12787,7 @@
       <c r="N232" s="9"/>
       <c r="O232" s="1"/>
     </row>
-    <row r="233" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A233" s="1"/>
       <c r="B233" s="31">
         <f t="shared" si="87"/>
@@ -12833,7 +12833,7 @@
       <c r="N233" s="9"/>
       <c r="O233" s="1"/>
     </row>
-    <row r="234" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A234" s="1"/>
       <c r="B234" s="31">
         <f t="shared" si="87"/>
@@ -12879,7 +12879,7 @@
       <c r="N234" s="9"/>
       <c r="O234" s="1"/>
     </row>
-    <row r="235" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A235" s="1"/>
       <c r="B235" s="31">
         <f t="shared" si="87"/>
@@ -12925,7 +12925,7 @@
       <c r="N235" s="9"/>
       <c r="O235" s="1"/>
     </row>
-    <row r="236" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A236" s="1"/>
       <c r="B236" s="31">
         <f t="shared" si="87"/>
@@ -12971,7 +12971,7 @@
       <c r="N236" s="9"/>
       <c r="O236" s="1"/>
     </row>
-    <row r="237" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A237" s="1"/>
       <c r="B237" s="31">
         <f t="shared" si="87"/>
@@ -13017,7 +13017,7 @@
       <c r="N237" s="9"/>
       <c r="O237" s="1"/>
     </row>
-    <row r="238" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A238" s="1"/>
       <c r="B238" s="31">
         <f t="shared" si="87"/>
@@ -13063,7 +13063,7 @@
       <c r="N238" s="9"/>
       <c r="O238" s="1"/>
     </row>
-    <row r="239" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A239" s="1"/>
       <c r="B239" s="31">
         <f t="shared" si="87"/>
@@ -13109,7 +13109,7 @@
       <c r="N239" s="9"/>
       <c r="O239" s="1"/>
     </row>
-    <row r="240" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A240" s="1"/>
       <c r="B240" s="31">
         <f t="shared" si="87"/>
@@ -13155,7 +13155,7 @@
       <c r="N240" s="9"/>
       <c r="O240" s="1"/>
     </row>
-    <row r="241" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A241" s="1"/>
       <c r="B241" s="31">
         <f t="shared" si="87"/>
@@ -13201,7 +13201,7 @@
       <c r="N241" s="9"/>
       <c r="O241" s="1"/>
     </row>
-    <row r="242" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A242" s="8"/>
       <c r="B242" s="31">
         <f t="shared" si="87"/>
@@ -13247,7 +13247,7 @@
       <c r="N242" s="9"/>
       <c r="O242" s="9"/>
     </row>
-    <row r="243" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A243" s="8"/>
       <c r="B243" s="31">
         <f t="shared" si="87"/>
@@ -13293,7 +13293,7 @@
       <c r="N243" s="9"/>
       <c r="O243" s="9"/>
     </row>
-    <row r="244" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A244" s="8"/>
       <c r="B244" s="31">
         <f t="shared" si="87"/>
@@ -13339,7 +13339,7 @@
       <c r="N244" s="9"/>
       <c r="O244" s="9"/>
     </row>
-    <row r="245" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A245" s="8"/>
       <c r="B245" s="31">
         <f t="shared" si="87"/>
@@ -13385,7 +13385,7 @@
       <c r="N245" s="9"/>
       <c r="O245" s="9"/>
     </row>
-    <row r="246" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A246" s="8"/>
       <c r="B246" s="31">
         <f t="shared" si="87"/>
@@ -13431,7 +13431,7 @@
       <c r="N246" s="9"/>
       <c r="O246" s="9"/>
     </row>
-    <row r="247" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A247" s="8"/>
       <c r="B247" s="31">
         <f t="shared" si="87"/>
@@ -13477,7 +13477,7 @@
       <c r="N247" s="9"/>
       <c r="O247" s="9"/>
     </row>
-    <row r="248" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A248" s="8"/>
       <c r="B248" s="31">
         <f t="shared" si="87"/>
@@ -13523,7 +13523,7 @@
       <c r="N248" s="9"/>
       <c r="O248" s="9"/>
     </row>
-    <row r="249" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A249" s="8"/>
       <c r="B249" s="31">
         <f t="shared" si="87"/>
@@ -13569,7 +13569,7 @@
       <c r="N249" s="9"/>
       <c r="O249" s="9"/>
     </row>
-    <row r="250" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A250" s="8"/>
       <c r="B250" s="31">
         <f t="shared" si="87"/>
@@ -13615,7 +13615,7 @@
       <c r="N250" s="9"/>
       <c r="O250" s="9"/>
     </row>
-    <row r="251" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A251" s="1"/>
       <c r="B251" s="31">
         <f t="shared" si="87"/>
@@ -13661,7 +13661,7 @@
       <c r="N251" s="9"/>
       <c r="O251" s="1"/>
     </row>
-    <row r="252" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A252" s="1"/>
       <c r="B252" s="31">
         <f t="shared" si="87"/>
@@ -13707,7 +13707,7 @@
       <c r="N252" s="9"/>
       <c r="O252" s="1"/>
     </row>
-    <row r="253" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A253" s="1"/>
       <c r="B253" s="31">
         <f t="shared" si="87"/>
@@ -13753,7 +13753,7 @@
       <c r="N253" s="9"/>
       <c r="O253" s="1"/>
     </row>
-    <row r="254" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A254" s="1"/>
       <c r="B254" s="31">
         <f t="shared" si="87"/>
@@ -13799,7 +13799,7 @@
       <c r="N254" s="9"/>
       <c r="O254" s="1"/>
     </row>
-    <row r="255" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A255" s="1"/>
       <c r="B255" s="31">
         <f t="shared" si="87"/>
@@ -13845,7 +13845,7 @@
       <c r="N255" s="9"/>
       <c r="O255" s="1"/>
     </row>
-    <row r="256" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A256" s="1"/>
       <c r="B256" s="31">
         <f t="shared" si="87"/>
@@ -13891,7 +13891,7 @@
       <c r="N256" s="9"/>
       <c r="O256" s="1"/>
     </row>
-    <row r="257" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A257" s="1"/>
       <c r="B257" s="31">
         <f t="shared" si="87"/>
@@ -13937,7 +13937,7 @@
       <c r="N257" s="9"/>
       <c r="O257" s="1"/>
     </row>
-    <row r="258" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A258" s="1"/>
       <c r="B258" s="31">
         <f t="shared" si="87"/>
@@ -13983,7 +13983,7 @@
       <c r="N258" s="9"/>
       <c r="O258" s="1"/>
     </row>
-    <row r="259" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A259" s="1"/>
       <c r="B259" s="31">
         <f t="shared" si="87"/>
@@ -14029,7 +14029,7 @@
       <c r="N259" s="9"/>
       <c r="O259" s="1"/>
     </row>
-    <row r="260" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A260" s="1"/>
       <c r="B260" s="31">
         <f t="shared" si="87"/>
@@ -14075,7 +14075,7 @@
       <c r="N260" s="9"/>
       <c r="O260" s="1"/>
     </row>
-    <row r="261" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A261" s="1"/>
       <c r="B261" s="31">
         <f t="shared" si="87"/>
@@ -14121,7 +14121,7 @@
       <c r="N261" s="9"/>
       <c r="O261" s="1"/>
     </row>
-    <row r="262" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A262" s="1"/>
       <c r="B262" s="31">
         <f t="shared" si="87"/>
@@ -14167,7 +14167,7 @@
       <c r="N262" s="9"/>
       <c r="O262" s="1"/>
     </row>
-    <row r="263" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A263" s="1"/>
       <c r="B263" s="31">
         <f t="shared" si="87"/>
@@ -14213,7 +14213,7 @@
       <c r="N263" s="9"/>
       <c r="O263" s="1"/>
     </row>
-    <row r="264" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A264" s="1"/>
       <c r="B264" s="31">
         <f t="shared" si="87"/>
@@ -14259,7 +14259,7 @@
       <c r="N264" s="9"/>
       <c r="O264" s="1"/>
     </row>
-    <row r="265" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A265" s="1"/>
       <c r="B265" s="31">
         <f t="shared" ref="B265:B293" si="119">+B264+1</f>
@@ -14305,7 +14305,7 @@
       <c r="N265" s="9"/>
       <c r="O265" s="1"/>
     </row>
-    <row r="266" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A266" s="1"/>
       <c r="B266" s="31">
         <f t="shared" si="119"/>
@@ -14351,7 +14351,7 @@
       <c r="N266" s="9"/>
       <c r="O266" s="1"/>
     </row>
-    <row r="267" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A267" s="1"/>
       <c r="B267" s="31">
         <f t="shared" si="119"/>
@@ -14397,7 +14397,7 @@
       <c r="N267" s="9"/>
       <c r="O267" s="1"/>
     </row>
-    <row r="268" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A268" s="1"/>
       <c r="B268" s="31">
         <f t="shared" si="119"/>
@@ -14443,7 +14443,7 @@
       <c r="N268" s="9"/>
       <c r="O268" s="1"/>
     </row>
-    <row r="269" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A269" s="1"/>
       <c r="B269" s="31">
         <f t="shared" si="119"/>
@@ -14489,7 +14489,7 @@
       <c r="N269" s="9"/>
       <c r="O269" s="1"/>
     </row>
-    <row r="270" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A270" s="1"/>
       <c r="B270" s="31">
         <f t="shared" si="119"/>
@@ -14535,7 +14535,7 @@
       <c r="N270" s="9"/>
       <c r="O270" s="1"/>
     </row>
-    <row r="271" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A271" s="1"/>
       <c r="B271" s="31">
         <f t="shared" si="119"/>
@@ -14581,7 +14581,7 @@
       <c r="N271" s="9"/>
       <c r="O271" s="1"/>
     </row>
-    <row r="272" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A272" s="1"/>
       <c r="B272" s="31">
         <f t="shared" si="119"/>
@@ -14627,7 +14627,7 @@
       <c r="N272" s="9"/>
       <c r="O272" s="1"/>
     </row>
-    <row r="273" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A273" s="1"/>
       <c r="B273" s="31">
         <f t="shared" si="119"/>
@@ -14673,7 +14673,7 @@
       <c r="N273" s="9"/>
       <c r="O273" s="1"/>
     </row>
-    <row r="274" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A274" s="1"/>
       <c r="B274" s="31">
         <f t="shared" si="119"/>
@@ -14719,7 +14719,7 @@
       <c r="N274" s="9"/>
       <c r="O274" s="1"/>
     </row>
-    <row r="275" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A275" s="1"/>
       <c r="B275" s="31">
         <f t="shared" si="119"/>
@@ -14765,7 +14765,7 @@
       <c r="N275" s="9"/>
       <c r="O275" s="1"/>
     </row>
-    <row r="276" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A276" s="1"/>
       <c r="B276" s="31">
         <f t="shared" si="119"/>
@@ -14811,7 +14811,7 @@
       <c r="N276" s="9"/>
       <c r="O276" s="1"/>
     </row>
-    <row r="277" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A277" s="1"/>
       <c r="B277" s="31">
         <f t="shared" si="119"/>
@@ -14857,7 +14857,7 @@
       <c r="N277" s="9"/>
       <c r="O277" s="1"/>
     </row>
-    <row r="278" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A278" s="1"/>
       <c r="B278" s="31">
         <f t="shared" si="119"/>
@@ -14903,7 +14903,7 @@
       <c r="N278" s="9"/>
       <c r="O278" s="1"/>
     </row>
-    <row r="279" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A279" s="1"/>
       <c r="B279" s="31">
         <f t="shared" si="119"/>
@@ -14949,7 +14949,7 @@
       <c r="N279" s="9"/>
       <c r="O279" s="1"/>
     </row>
-    <row r="280" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A280" s="1"/>
       <c r="B280" s="31">
         <f t="shared" si="119"/>
@@ -14995,7 +14995,7 @@
       <c r="N280" s="9"/>
       <c r="O280" s="1"/>
     </row>
-    <row r="281" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A281" s="1"/>
       <c r="B281" s="31">
         <f t="shared" si="119"/>
@@ -15041,7 +15041,7 @@
       <c r="N281" s="9"/>
       <c r="O281" s="1"/>
     </row>
-    <row r="282" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A282" s="1"/>
       <c r="B282" s="31">
         <f t="shared" si="119"/>
@@ -15087,7 +15087,7 @@
       <c r="N282" s="9"/>
       <c r="O282" s="1"/>
     </row>
-    <row r="283" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A283" s="1"/>
       <c r="B283" s="31">
         <f t="shared" si="119"/>
@@ -15133,7 +15133,7 @@
       <c r="N283" s="9"/>
       <c r="O283" s="1"/>
     </row>
-    <row r="284" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A284" s="1"/>
       <c r="B284" s="31">
         <f t="shared" si="119"/>
@@ -15179,7 +15179,7 @@
       <c r="N284" s="9"/>
       <c r="O284" s="1"/>
     </row>
-    <row r="285" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A285" s="1"/>
       <c r="B285" s="31">
         <f t="shared" si="119"/>
@@ -15225,7 +15225,7 @@
       <c r="N285" s="9"/>
       <c r="O285" s="1"/>
     </row>
-    <row r="286" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A286" s="1"/>
       <c r="B286" s="31">
         <f t="shared" si="119"/>
@@ -15271,7 +15271,7 @@
       <c r="N286" s="9"/>
       <c r="O286" s="1"/>
     </row>
-    <row r="287" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A287" s="1"/>
       <c r="B287" s="31">
         <f t="shared" si="119"/>
@@ -15317,7 +15317,7 @@
       <c r="N287" s="9"/>
       <c r="O287" s="1"/>
     </row>
-    <row r="288" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A288" s="1"/>
       <c r="B288" s="31">
         <f t="shared" si="119"/>
@@ -15363,7 +15363,7 @@
       <c r="N288" s="9"/>
       <c r="O288" s="1"/>
     </row>
-    <row r="289" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A289" s="1"/>
       <c r="B289" s="31">
         <f t="shared" si="119"/>
@@ -15409,7 +15409,7 @@
       <c r="N289" s="9"/>
       <c r="O289" s="1"/>
     </row>
-    <row r="290" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A290" s="1"/>
       <c r="B290" s="31">
         <f t="shared" si="119"/>
@@ -15455,7 +15455,7 @@
       <c r="N290" s="9"/>
       <c r="O290" s="1"/>
     </row>
-    <row r="291" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A291" s="1"/>
       <c r="B291" s="31">
         <f t="shared" si="119"/>
@@ -15501,7 +15501,7 @@
       <c r="N291" s="9"/>
       <c r="O291" s="1"/>
     </row>
-    <row r="292" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A292" s="1"/>
       <c r="B292" s="31">
         <f t="shared" si="119"/>
@@ -15547,7 +15547,7 @@
       <c r="N292" s="9"/>
       <c r="O292" s="1"/>
     </row>
-    <row r="293" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A293" s="1"/>
       <c r="B293" s="31">
         <f t="shared" si="119"/>
@@ -15593,7 +15593,7 @@
       <c r="N293" s="9"/>
       <c r="O293" s="1"/>
     </row>
-    <row r="294" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A294" s="1"/>
       <c r="B294" s="31">
         <f t="shared" ref="B294:B295" si="126">+B293+1</f>
@@ -15639,7 +15639,7 @@
       <c r="N294" s="9"/>
       <c r="O294" s="1"/>
     </row>
-    <row r="295" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:15" ht="16.5" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A295" s="1"/>
       <c r="B295" s="31">
         <f t="shared" si="126"/>
@@ -15685,7 +15685,7 @@
       <c r="N295" s="9"/>
       <c r="O295" s="1"/>
     </row>
-    <row r="296" spans="1:15" ht="16.5" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:15" ht="16.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A296" s="1"/>
       <c r="B296" s="31">
         <f t="shared" ref="B296:B359" si="130">+B295+1</f>
@@ -15731,7 +15731,7 @@
       <c r="N296" s="9"/>
       <c r="O296" s="1"/>
     </row>
-    <row r="297" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" s="8"/>
       <c r="B297" s="31">
         <f t="shared" si="130"/>
@@ -15777,7 +15777,7 @@
       <c r="N297" s="1"/>
       <c r="O297" s="1"/>
     </row>
-    <row r="298" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" s="8"/>
       <c r="B298" s="31">
         <f t="shared" si="130"/>
@@ -15822,7 +15822,7 @@
       <c r="N298" s="1"/>
       <c r="O298" s="1"/>
     </row>
-    <row r="299" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" s="8"/>
       <c r="B299" s="31">
         <f t="shared" si="130"/>
@@ -15867,7 +15867,7 @@
       <c r="N299" s="1"/>
       <c r="O299" s="1"/>
     </row>
-    <row r="300" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" s="8"/>
       <c r="B300" s="31">
         <f t="shared" si="130"/>
@@ -16092,7 +16092,7 @@
       <c r="N304" s="7"/>
       <c r="O304" s="7"/>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="7"/>
       <c r="B305" s="31">
         <f t="shared" si="130"/>
@@ -16137,7 +16137,7 @@
       <c r="N305" s="7"/>
       <c r="O305" s="7"/>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="7"/>
       <c r="B306" s="31">
         <f t="shared" si="130"/>
@@ -16182,7 +16182,7 @@
       <c r="N306" s="7"/>
       <c r="O306" s="7"/>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="7"/>
       <c r="B307" s="31">
         <f t="shared" si="130"/>
@@ -16227,7 +16227,7 @@
       <c r="N307" s="7"/>
       <c r="O307" s="7"/>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="7"/>
       <c r="B308" s="31">
         <f t="shared" si="130"/>
@@ -16272,7 +16272,7 @@
       <c r="N308" s="7"/>
       <c r="O308" s="7"/>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="7"/>
       <c r="B309" s="31">
         <f t="shared" si="130"/>
@@ -16317,7 +16317,7 @@
       <c r="N309" s="7"/>
       <c r="O309" s="7"/>
     </row>
-    <row r="310" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" s="1"/>
       <c r="B310" s="31">
         <f t="shared" si="130"/>
@@ -16362,7 +16362,7 @@
       <c r="N310" s="1"/>
       <c r="O310" s="1"/>
     </row>
-    <row r="311" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" s="1"/>
       <c r="B311" s="31">
         <f t="shared" si="130"/>
@@ -16407,7 +16407,7 @@
       <c r="N311" s="1"/>
       <c r="O311" s="1"/>
     </row>
-    <row r="312" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" s="1"/>
       <c r="B312" s="31">
         <f t="shared" si="130"/>
@@ -16452,7 +16452,7 @@
       <c r="N312" s="1"/>
       <c r="O312" s="1"/>
     </row>
-    <row r="313" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" s="1"/>
       <c r="B313" s="31">
         <f t="shared" si="130"/>
@@ -16497,7 +16497,7 @@
       <c r="N313" s="1"/>
       <c r="O313" s="1"/>
     </row>
-    <row r="314" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" s="1"/>
       <c r="B314" s="31">
         <f t="shared" si="130"/>
@@ -16542,7 +16542,7 @@
       <c r="N314" s="1"/>
       <c r="O314" s="1"/>
     </row>
-    <row r="315" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" s="1"/>
       <c r="B315" s="31">
         <f t="shared" si="130"/>
@@ -16587,7 +16587,7 @@
       <c r="N315" s="1"/>
       <c r="O315" s="1"/>
     </row>
-    <row r="316" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" s="1"/>
       <c r="B316" s="31">
         <f t="shared" si="130"/>
@@ -16632,7 +16632,7 @@
       <c r="N316" s="1"/>
       <c r="O316" s="1"/>
     </row>
-    <row r="317" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" s="1"/>
       <c r="B317" s="31">
         <f t="shared" si="130"/>
@@ -16677,7 +16677,7 @@
       <c r="N317" s="1"/>
       <c r="O317" s="1"/>
     </row>
-    <row r="318" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" s="1"/>
       <c r="B318" s="31">
         <f t="shared" si="130"/>
@@ -16722,7 +16722,7 @@
       <c r="N318" s="1"/>
       <c r="O318" s="1"/>
     </row>
-    <row r="319" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" s="1"/>
       <c r="B319" s="31">
         <f t="shared" si="130"/>
@@ -16767,7 +16767,7 @@
       <c r="N319" s="1"/>
       <c r="O319" s="1"/>
     </row>
-    <row r="320" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" s="1"/>
       <c r="B320" s="31">
         <f t="shared" si="130"/>
@@ -16812,7 +16812,7 @@
       <c r="N320" s="1"/>
       <c r="O320" s="1"/>
     </row>
-    <row r="321" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" s="1"/>
       <c r="B321" s="31">
         <f t="shared" si="130"/>
@@ -16857,7 +16857,7 @@
       <c r="N321" s="1"/>
       <c r="O321" s="1"/>
     </row>
-    <row r="322" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" s="1"/>
       <c r="B322" s="31">
         <f t="shared" si="130"/>
@@ -16902,7 +16902,7 @@
       <c r="N322" s="1"/>
       <c r="O322" s="1"/>
     </row>
-    <row r="323" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" s="1"/>
       <c r="B323" s="31">
         <f t="shared" si="130"/>
@@ -16947,7 +16947,7 @@
       <c r="N323" s="1"/>
       <c r="O323" s="1"/>
     </row>
-    <row r="324" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" s="1"/>
       <c r="B324" s="31">
         <f t="shared" si="130"/>
@@ -16992,7 +16992,7 @@
       <c r="N324" s="1"/>
       <c r="O324" s="1"/>
     </row>
-    <row r="325" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" s="1"/>
       <c r="B325" s="31">
         <f t="shared" si="130"/>
@@ -17037,7 +17037,7 @@
       <c r="N325" s="1"/>
       <c r="O325" s="1"/>
     </row>
-    <row r="326" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" s="1"/>
       <c r="B326" s="31">
         <f t="shared" si="130"/>
@@ -17082,7 +17082,7 @@
       <c r="N326" s="1"/>
       <c r="O326" s="1"/>
     </row>
-    <row r="327" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" s="1"/>
       <c r="B327" s="31">
         <f t="shared" si="130"/>
@@ -17127,7 +17127,7 @@
       <c r="N327" s="1"/>
       <c r="O327" s="1"/>
     </row>
-    <row r="328" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" s="1"/>
       <c r="B328" s="31">
         <f t="shared" si="130"/>
@@ -17172,7 +17172,7 @@
       <c r="N328" s="1"/>
       <c r="O328" s="1"/>
     </row>
-    <row r="329" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" s="1"/>
       <c r="B329" s="31">
         <f t="shared" si="130"/>
@@ -17217,7 +17217,7 @@
       <c r="N329" s="1"/>
       <c r="O329" s="1"/>
     </row>
-    <row r="330" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" s="1"/>
       <c r="B330" s="31">
         <f t="shared" si="130"/>
@@ -17262,7 +17262,7 @@
       <c r="N330" s="1"/>
       <c r="O330" s="1"/>
     </row>
-    <row r="331" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" s="1"/>
       <c r="B331" s="31">
         <f t="shared" si="130"/>
@@ -17307,7 +17307,7 @@
       <c r="N331" s="1"/>
       <c r="O331" s="1"/>
     </row>
-    <row r="332" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" s="1"/>
       <c r="B332" s="31">
         <f t="shared" si="130"/>
@@ -17352,7 +17352,7 @@
       <c r="N332" s="1"/>
       <c r="O332" s="1"/>
     </row>
-    <row r="333" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" s="1"/>
       <c r="B333" s="31">
         <f t="shared" si="130"/>
@@ -17397,7 +17397,7 @@
       <c r="N333" s="1"/>
       <c r="O333" s="1"/>
     </row>
-    <row r="334" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" s="1"/>
       <c r="B334" s="31">
         <f t="shared" si="130"/>
@@ -17442,7 +17442,7 @@
       <c r="N334" s="1"/>
       <c r="O334" s="1"/>
     </row>
-    <row r="335" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" s="1"/>
       <c r="B335" s="31">
         <f t="shared" si="130"/>
@@ -17487,7 +17487,7 @@
       <c r="N335" s="1"/>
       <c r="O335" s="1"/>
     </row>
-    <row r="336" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" s="1"/>
       <c r="B336" s="31">
         <f t="shared" si="130"/>
@@ -17532,7 +17532,7 @@
       <c r="N336" s="1"/>
       <c r="O336" s="1"/>
     </row>
-    <row r="337" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" s="1"/>
       <c r="B337" s="31">
         <f t="shared" si="130"/>
@@ -17577,7 +17577,7 @@
       <c r="N337" s="1"/>
       <c r="O337" s="1"/>
     </row>
-    <row r="338" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" s="1"/>
       <c r="B338" s="31">
         <f t="shared" si="130"/>
@@ -17622,7 +17622,7 @@
       <c r="N338" s="1"/>
       <c r="O338" s="1"/>
     </row>
-    <row r="339" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" s="1"/>
       <c r="B339" s="31">
         <f t="shared" si="130"/>
@@ -17667,7 +17667,7 @@
       <c r="N339" s="1"/>
       <c r="O339" s="1"/>
     </row>
-    <row r="340" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" s="1"/>
       <c r="B340" s="31">
         <f t="shared" si="130"/>
@@ -17712,7 +17712,7 @@
       <c r="N340" s="1"/>
       <c r="O340" s="1"/>
     </row>
-    <row r="341" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" s="1"/>
       <c r="B341" s="31">
         <f t="shared" si="130"/>
@@ -17757,7 +17757,7 @@
       <c r="N341" s="1"/>
       <c r="O341" s="1"/>
     </row>
-    <row r="342" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" s="1"/>
       <c r="B342" s="31">
         <f t="shared" si="130"/>
@@ -17802,7 +17802,7 @@
       <c r="N342" s="1"/>
       <c r="O342" s="1"/>
     </row>
-    <row r="343" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" s="1"/>
       <c r="B343" s="31">
         <f t="shared" si="130"/>
@@ -17847,7 +17847,7 @@
       <c r="N343" s="1"/>
       <c r="O343" s="1"/>
     </row>
-    <row r="344" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" s="1"/>
       <c r="B344" s="31">
         <f t="shared" si="130"/>
@@ -17892,7 +17892,7 @@
       <c r="N344" s="1"/>
       <c r="O344" s="1"/>
     </row>
-    <row r="345" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" s="1"/>
       <c r="B345" s="31">
         <f t="shared" si="130"/>
@@ -17937,7 +17937,7 @@
       <c r="N345" s="1"/>
       <c r="O345" s="1"/>
     </row>
-    <row r="346" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" s="1"/>
       <c r="B346" s="31">
         <f t="shared" si="130"/>
@@ -17982,7 +17982,7 @@
       <c r="N346" s="1"/>
       <c r="O346" s="1"/>
     </row>
-    <row r="347" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" s="1"/>
       <c r="B347" s="31">
         <f t="shared" si="130"/>
@@ -18027,7 +18027,7 @@
       <c r="N347" s="1"/>
       <c r="O347" s="1"/>
     </row>
-    <row r="348" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" s="1"/>
       <c r="B348" s="31">
         <f t="shared" si="130"/>
@@ -18072,7 +18072,7 @@
       <c r="N348" s="1"/>
       <c r="O348" s="1"/>
     </row>
-    <row r="349" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" s="1"/>
       <c r="B349" s="31">
         <f t="shared" si="130"/>
@@ -18117,7 +18117,7 @@
       <c r="N349" s="1"/>
       <c r="O349" s="1"/>
     </row>
-    <row r="350" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" s="1"/>
       <c r="B350" s="31">
         <f t="shared" si="130"/>
@@ -18162,7 +18162,7 @@
       <c r="N350" s="1"/>
       <c r="O350" s="1"/>
     </row>
-    <row r="351" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" s="1"/>
       <c r="B351" s="31">
         <f t="shared" si="130"/>
@@ -18207,7 +18207,7 @@
       <c r="N351" s="1"/>
       <c r="O351" s="1"/>
     </row>
-    <row r="352" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" s="1"/>
       <c r="B352" s="31">
         <f t="shared" si="130"/>
@@ -18252,7 +18252,7 @@
       <c r="N352" s="1"/>
       <c r="O352" s="1"/>
     </row>
-    <row r="353" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" s="1"/>
       <c r="B353" s="31">
         <f t="shared" si="130"/>
@@ -18297,7 +18297,7 @@
       <c r="N353" s="1"/>
       <c r="O353" s="1"/>
     </row>
-    <row r="354" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" s="1"/>
       <c r="B354" s="31">
         <f t="shared" si="130"/>
@@ -18342,7 +18342,7 @@
       <c r="N354" s="1"/>
       <c r="O354" s="1"/>
     </row>
-    <row r="355" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" s="1"/>
       <c r="B355" s="31">
         <f t="shared" si="130"/>
@@ -18387,7 +18387,7 @@
       <c r="N355" s="1"/>
       <c r="O355" s="1"/>
     </row>
-    <row r="356" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" s="1"/>
       <c r="B356" s="31">
         <f t="shared" si="130"/>
@@ -18432,7 +18432,7 @@
       <c r="N356" s="1"/>
       <c r="O356" s="1"/>
     </row>
-    <row r="357" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" s="1"/>
       <c r="B357" s="31">
         <f t="shared" si="130"/>
@@ -18477,7 +18477,7 @@
       <c r="N357" s="1"/>
       <c r="O357" s="1"/>
     </row>
-    <row r="358" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" s="1"/>
       <c r="B358" s="31">
         <f t="shared" si="130"/>
@@ -18522,7 +18522,7 @@
       <c r="N358" s="1"/>
       <c r="O358" s="1"/>
     </row>
-    <row r="359" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" s="1"/>
       <c r="B359" s="31">
         <f t="shared" si="130"/>
@@ -18566,7 +18566,7 @@
       <c r="N359" s="1"/>
       <c r="O359" s="1"/>
     </row>
-    <row r="360" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" s="1"/>
       <c r="B360" s="31">
         <f t="shared" ref="B360:B374" si="135">+B359+1</f>
@@ -18654,7 +18654,7 @@
       <c r="N361" s="1"/>
       <c r="O361" s="1"/>
     </row>
-    <row r="362" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" s="1"/>
       <c r="B362" s="31">
         <f t="shared" si="135"/>
@@ -18698,7 +18698,7 @@
       <c r="N362" s="1"/>
       <c r="O362" s="1"/>
     </row>
-    <row r="363" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363" s="1"/>
       <c r="B363" s="31">
         <f t="shared" si="135"/>
@@ -18742,7 +18742,7 @@
       <c r="N363" s="1"/>
       <c r="O363" s="1"/>
     </row>
-    <row r="364" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364" s="1"/>
       <c r="B364" s="31">
         <f t="shared" si="135"/>
@@ -18786,7 +18786,7 @@
       <c r="N364" s="1"/>
       <c r="O364" s="1"/>
     </row>
-    <row r="365" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" s="1"/>
       <c r="B365" s="31">
         <f t="shared" si="135"/>
@@ -18830,7 +18830,7 @@
       <c r="N365" s="1"/>
       <c r="O365" s="1"/>
     </row>
-    <row r="366" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" s="1"/>
       <c r="B366" s="31">
         <f t="shared" si="135"/>
@@ -18874,7 +18874,7 @@
       <c r="N366" s="1"/>
       <c r="O366" s="1"/>
     </row>
-    <row r="367" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367" s="1"/>
       <c r="B367" s="31">
         <f t="shared" si="135"/>
@@ -18918,7 +18918,7 @@
       <c r="N367" s="1"/>
       <c r="O367" s="1"/>
     </row>
-    <row r="368" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" s="1"/>
       <c r="B368" s="31">
         <f t="shared" si="135"/>
@@ -18962,7 +18962,7 @@
       <c r="N368" s="1"/>
       <c r="O368" s="1"/>
     </row>
-    <row r="369" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" s="1"/>
       <c r="B369" s="31">
         <f t="shared" si="135"/>
@@ -19006,7 +19006,7 @@
       <c r="N369" s="1"/>
       <c r="O369" s="1"/>
     </row>
-    <row r="370" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" s="1"/>
       <c r="B370" s="31">
         <f t="shared" si="135"/>
@@ -19050,7 +19050,7 @@
       <c r="N370" s="1"/>
       <c r="O370" s="1"/>
     </row>
-    <row r="371" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" s="1"/>
       <c r="B371" s="31">
         <f t="shared" si="135"/>
@@ -19094,7 +19094,7 @@
       <c r="N371" s="1"/>
       <c r="O371" s="1"/>
     </row>
-    <row r="372" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" s="1"/>
       <c r="B372" s="31">
         <f t="shared" si="135"/>
@@ -19138,7 +19138,7 @@
       <c r="N372" s="1"/>
       <c r="O372" s="1"/>
     </row>
-    <row r="373" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" s="1"/>
       <c r="B373" s="31">
         <f t="shared" si="135"/>
@@ -19182,7 +19182,7 @@
       <c r="N373" s="1"/>
       <c r="O373" s="1"/>
     </row>
-    <row r="374" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" s="1"/>
       <c r="B374" s="31">
         <f t="shared" si="135"/>
@@ -19226,7 +19226,7 @@
       <c r="N374" s="1"/>
       <c r="O374" s="1"/>
     </row>
-    <row r="375" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" s="1"/>
       <c r="B375" s="1"/>
       <c r="C375" s="4"/>
@@ -19238,7 +19238,7 @@
       <c r="N375" s="1"/>
       <c r="O375" s="1"/>
     </row>
-    <row r="376" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" s="1"/>
       <c r="B376" s="1"/>
       <c r="C376" s="4"/>
@@ -19250,7 +19250,7 @@
       <c r="N376" s="1"/>
       <c r="O376" s="1"/>
     </row>
-    <row r="377" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" s="1"/>
       <c r="B377" s="1"/>
       <c r="C377" s="4"/>
@@ -19262,7 +19262,7 @@
       <c r="N377" s="1"/>
       <c r="O377" s="1"/>
     </row>
-    <row r="378" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" s="1"/>
       <c r="B378" s="1"/>
       <c r="C378" s="4"/>
@@ -19274,7 +19274,7 @@
       <c r="N378" s="1"/>
       <c r="O378" s="1"/>
     </row>
-    <row r="379" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" s="1"/>
       <c r="B379" s="1"/>
       <c r="C379" s="4"/>
@@ -19286,7 +19286,7 @@
       <c r="N379" s="1"/>
       <c r="O379" s="1"/>
     </row>
-    <row r="380" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" s="1"/>
       <c r="B380" s="1"/>
       <c r="C380" s="4"/>
@@ -19298,7 +19298,7 @@
       <c r="N380" s="1"/>
       <c r="O380" s="1"/>
     </row>
-    <row r="381" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" s="1"/>
       <c r="B381" s="1"/>
       <c r="C381" s="4"/>
@@ -19310,7 +19310,7 @@
       <c r="N381" s="1"/>
       <c r="O381" s="1"/>
     </row>
-    <row r="382" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" s="1"/>
       <c r="B382" s="1"/>
       <c r="C382" s="4"/>
@@ -19322,7 +19322,7 @@
       <c r="N382" s="1"/>
       <c r="O382" s="1"/>
     </row>
-    <row r="383" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" s="1"/>
       <c r="B383" s="1"/>
       <c r="C383" s="4"/>
@@ -19334,7 +19334,7 @@
       <c r="N383" s="1"/>
       <c r="O383" s="1"/>
     </row>
-    <row r="384" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" s="1"/>
       <c r="B384" s="1"/>
       <c r="C384" s="4"/>
@@ -19346,7 +19346,7 @@
       <c r="N384" s="1"/>
       <c r="O384" s="1"/>
     </row>
-    <row r="385" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" s="1"/>
       <c r="B385" s="1"/>
       <c r="C385" s="4"/>
@@ -19358,7 +19358,7 @@
       <c r="N385" s="1"/>
       <c r="O385" s="1"/>
     </row>
-    <row r="386" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" s="1"/>
       <c r="B386" s="1"/>
       <c r="C386" s="4"/>
@@ -19370,7 +19370,7 @@
       <c r="N386" s="1"/>
       <c r="O386" s="1"/>
     </row>
-    <row r="387" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" s="1"/>
       <c r="B387" s="1"/>
       <c r="C387" s="4"/>
@@ -19382,7 +19382,7 @@
       <c r="N387" s="1"/>
       <c r="O387" s="1"/>
     </row>
-    <row r="388" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" s="1"/>
       <c r="B388" s="1"/>
       <c r="C388" s="4"/>
@@ -19394,7 +19394,7 @@
       <c r="N388" s="1"/>
       <c r="O388" s="1"/>
     </row>
-    <row r="389" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" s="1"/>
       <c r="B389" s="1"/>
       <c r="C389" s="4"/>
@@ -19406,7 +19406,7 @@
       <c r="N389" s="1"/>
       <c r="O389" s="1"/>
     </row>
-    <row r="390" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:15" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" s="1"/>
       <c r="B390" s="1"/>
       <c r="C390" s="4"/>
@@ -29182,7 +29182,13 @@
       <c r="O1097" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="C5:N390" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}"/>
+  <autoFilter ref="C5:N390" xr:uid="{B112AD15-80BE-4F57-9D44-7F3B8C4B4536}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Contacts"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="C3:E3"/>
   </mergeCells>

</xml_diff>